<commit_message>
Fix .NET 8 auto-property memory layout bug in Item struct
</commit_message>
<xml_diff>
--- a/ARM Functions/Ability Edits/Electropyresis.xlsx
+++ b/ARM Functions/Ability Edits/Electropyresis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\ROM\3ds\Modded ROM\USUM ARM research\Ability Edits\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\ROM\3ds\USUM ARM research\Ability Edits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877D5187-E447-4D89-BCE7-68D161D53ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FFBA8F-9D65-490A-8D20-4B041D5E95A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{DFD0B34E-FAAD-4BE6-8FC0-3053B30C3017}"/>
+    <workbookView xWindow="-16457" yWindow="0" windowWidth="16457" windowHeight="17914" xr2:uid="{DFD0B34E-FAAD-4BE6-8FC0-3053B30C3017}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="215">
   <si>
     <t>mov r1, r4</t>
   </si>
@@ -688,7 +688,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -705,16 +705,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <color theme="1"/>
+      <name val="Cascadia Code"/>
+      <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Cambria"/>
-      <family val="1"/>
+      <name val="Cascadia Code"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Cascadia Code"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="6">
@@ -761,21 +767,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1111,1207 +1123,1205 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52D5FF14-B243-47B9-B921-E1E0A4F7D67F}">
   <dimension ref="A1:O173"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15.9"/>
   <cols>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.86328125" customWidth="1"/>
+    <col min="2" max="2" width="9.35546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.78515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:15">
+      <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A3" s="4" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="8"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="8" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15">
       <c r="A4" t="str">
         <f t="shared" ref="A4:A7" si="0">DEC2HEX(HEX2DEC(A3)+4,8)</f>
         <v>000FE5CC</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>000FE5D0</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>000FE5D4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>000FE5D8</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="C8" s="1"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A9" s="3" t="s">
+    <row r="8" spans="1:15">
+      <c r="C8" s="10"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" t="str">
         <f>DEC2HEX(HEX2DEC(A7)+4,8)</f>
         <v>000FE5DC</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15">
       <c r="A11" t="str">
         <f t="shared" ref="A11" si="1">DEC2HEX(HEX2DEC(A10)+4,8)</f>
         <v>000FE5E0</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="O11" s="4"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="F11" s="2"/>
+      <c r="O11" s="2"/>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" t="str">
         <f t="shared" ref="A12" si="2">DEC2HEX(HEX2DEC(A11)+4,8)</f>
         <v>000FE5E4</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A13" s="5" t="str">
+    <row r="13" spans="1:15">
+      <c r="A13" s="3" t="str">
         <f t="shared" ref="A13" si="3">DEC2HEX(HEX2DEC(A12)+4,8)</f>
         <v>000FE5E8</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A14" s="5" t="str">
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" s="3" t="str">
         <f t="shared" ref="A14" si="4">DEC2HEX(HEX2DEC(A13)+4,8)</f>
         <v>000FE5EC</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="D14" s="5"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A15" s="5" t="str">
+      <c r="D14" s="12"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" s="3" t="str">
         <f t="shared" ref="A15" si="5">DEC2HEX(HEX2DEC(A14)+4,8)</f>
         <v>000FE5F0</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="F15" s="4"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A16" s="5" t="str">
+      <c r="D15" s="12"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" s="3" t="str">
         <f t="shared" ref="A16" si="6">DEC2HEX(HEX2DEC(A15)+4,8)</f>
         <v>000FE5F4</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="C16" s="5" t="str">
+      <c r="C16" s="12" t="str">
         <f>_xlfn.CONCAT("bne 0x",A34)</f>
         <v>bne 0x000FE63C</v>
       </c>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A17" s="7" t="str">
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="4" t="str">
         <f t="shared" ref="A17" si="7">DEC2HEX(HEX2DEC(A16)+4,8)</f>
         <v>000FE5F8</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A18" s="7" t="str">
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="4" t="str">
         <f t="shared" ref="A18" si="8">DEC2HEX(HEX2DEC(A17)+4,8)</f>
         <v>000FE5FC</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="D18" s="7"/>
-      <c r="F18" s="4"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A19" s="7" t="str">
+      <c r="D18" s="15"/>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="4" t="str">
         <f t="shared" ref="A19" si="9">DEC2HEX(HEX2DEC(A18)+4,8)</f>
         <v>000FE600</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A20" s="9" t="str">
+      <c r="D19" s="15"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="5" t="str">
         <f t="shared" ref="A20" si="10">DEC2HEX(HEX2DEC(A19)+4,8)</f>
         <v>000FE604</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A21" s="9" t="str">
+    <row r="21" spans="1:8">
+      <c r="A21" s="5" t="str">
         <f t="shared" ref="A21" si="11">DEC2HEX(HEX2DEC(A20)+4,8)</f>
         <v>000FE608</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="F21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A22" s="9" t="str">
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="5" t="str">
         <f t="shared" ref="A22" si="12">DEC2HEX(HEX2DEC(A21)+4,8)</f>
         <v>000FE60C</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A23" s="9" t="str">
+    <row r="23" spans="1:8">
+      <c r="A23" s="5" t="str">
         <f t="shared" ref="A23" si="13">DEC2HEX(HEX2DEC(A22)+4,8)</f>
         <v>000FE610</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="17" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A24" s="9" t="str">
+    <row r="24" spans="1:8">
+      <c r="A24" s="5" t="str">
         <f t="shared" ref="A24" si="14">DEC2HEX(HEX2DEC(A23)+4,8)</f>
         <v>000FE614</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="C24" s="9" t="str">
+      <c r="C24" s="16" t="str">
         <f>_xlfn.CONCAT("beq 0x",A$34)</f>
         <v>beq 0x000FE63C</v>
       </c>
-      <c r="D24" s="9"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A25" s="11" t="str">
+      <c r="D24" s="16"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="6" t="str">
         <f t="shared" ref="A25" si="15">DEC2HEX(HEX2DEC(A24)+4,8)</f>
         <v>000FE618</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="18" t="s">
         <v>208</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A26" s="11" t="str">
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="6" t="str">
         <f t="shared" ref="A26" si="16">DEC2HEX(HEX2DEC(A25)+4,8)</f>
         <v>000FE61C</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="D26" s="12" t="s">
+      <c r="D26" s="18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A27" s="11" t="str">
+    <row r="27" spans="1:8">
+      <c r="A27" s="6" t="str">
         <f t="shared" ref="A27" si="17">DEC2HEX(HEX2DEC(A26)+4,8)</f>
         <v>000FE620</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A28" s="11" t="str">
+    <row r="28" spans="1:8">
+      <c r="A28" s="6" t="str">
         <f t="shared" ref="A28" si="18">DEC2HEX(HEX2DEC(A27)+4,8)</f>
         <v>000FE624</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="19" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A29" s="11" t="str">
+    <row r="29" spans="1:8">
+      <c r="A29" s="6" t="str">
         <f t="shared" ref="A29" si="19">DEC2HEX(HEX2DEC(A28)+4,8)</f>
         <v>000FE628</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C29" s="11" t="str">
+      <c r="C29" s="19" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$34)</f>
         <v>bne 0x000FE63C</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="19" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:8">
       <c r="A30" t="str">
         <f t="shared" ref="A30" si="20">DEC2HEX(HEX2DEC(A29)+4,8)</f>
         <v>000FE62C</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:8">
       <c r="A31" t="str">
         <f t="shared" ref="A31" si="21">DEC2HEX(HEX2DEC(A30)+4,8)</f>
         <v>000FE630</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:8">
       <c r="A32" t="str">
         <f t="shared" ref="A32" si="22">DEC2HEX(HEX2DEC(A31)+4,8)</f>
         <v>000FE634</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="4" t="str">
+      <c r="C32" s="8" t="str">
         <f>SUBSTITUTE(C10,"push","pop")</f>
         <v>pop {r4, lr}</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:4">
       <c r="A33" t="str">
         <f t="shared" ref="A33" si="23">DEC2HEX(HEX2DEC(A32)+4,8)</f>
         <v>000FE638</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:4">
       <c r="A34" t="str">
         <f t="shared" ref="A34" si="24">DEC2HEX(HEX2DEC(A33)+4,8)</f>
         <v>000FE63C</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C34" s="4" t="str">
+      <c r="C34" s="8" t="str">
         <f>SUBSTITUTE(C32,"lr","pc")</f>
         <v>pop {r4, pc}</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C35" s="1"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A36" s="3" t="s">
+    <row r="35" spans="1:4">
+      <c r="C35" s="10"/>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="1"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C36" s="10"/>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" t="str">
         <f>DEC2HEX(HEX2DEC(A34)+4,8)</f>
         <v>000FE640</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:4">
       <c r="A38" t="str">
         <f t="shared" ref="A38" si="25">DEC2HEX(HEX2DEC(A37)+4,8)</f>
         <v>000FE644</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:4">
       <c r="A39" t="str">
         <f t="shared" ref="A39" si="26">DEC2HEX(HEX2DEC(A38)+4,8)</f>
         <v>000FE648</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A40" s="7" t="str">
+    <row r="40" spans="1:4">
+      <c r="A40" s="4" t="str">
         <f t="shared" ref="A40" si="27">DEC2HEX(HEX2DEC(A39)+4,8)</f>
         <v>000FE64C</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="15" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A41" s="7" t="str">
+    <row r="41" spans="1:4">
+      <c r="A41" s="4" t="str">
         <f t="shared" ref="A41" si="28">DEC2HEX(HEX2DEC(A40)+4,8)</f>
         <v>000FE650</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="D41" s="7"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A42" s="7" t="str">
+      <c r="D41" s="15"/>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="4" t="str">
         <f t="shared" ref="A42" si="29">DEC2HEX(HEX2DEC(A41)+4,8)</f>
         <v>000FE654</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C42" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="7"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A43" s="7" t="str">
+      <c r="D42" s="15"/>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="4" t="str">
         <f t="shared" ref="A43" si="30">DEC2HEX(HEX2DEC(A42)+4,8)</f>
         <v>000FE658</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="C43" s="8" t="str">
+      <c r="C43" s="14" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$54)</f>
         <v>bne 0x000FE684</v>
       </c>
-      <c r="D43" s="7"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A44" s="5" t="str">
+      <c r="D43" s="15"/>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="3" t="str">
         <f t="shared" ref="A44" si="31">DEC2HEX(HEX2DEC(A43)+4,8)</f>
         <v>000FE65C</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D44" s="5"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A45" s="5" t="str">
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="3" t="str">
         <f t="shared" ref="A45" si="32">DEC2HEX(HEX2DEC(A44)+4,8)</f>
         <v>000FE660</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="5"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A46" s="5" t="str">
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="3" t="str">
         <f t="shared" ref="A46" si="33">DEC2HEX(HEX2DEC(A45)+4,8)</f>
         <v>000FE664</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="D46" s="5"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A47" s="5" t="str">
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="3" t="str">
         <f t="shared" ref="A47" si="34">DEC2HEX(HEX2DEC(A46)+4,8)</f>
         <v>000FE668</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D47" s="5"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A48" s="5" t="str">
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="3" t="str">
         <f t="shared" ref="A48" si="35">DEC2HEX(HEX2DEC(A47)+4,8)</f>
         <v>000FE66C</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="D48" s="12" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A49" s="5" t="str">
+    <row r="49" spans="1:4">
+      <c r="A49" s="3" t="str">
         <f t="shared" ref="A49" si="36">DEC2HEX(HEX2DEC(A48)+4,8)</f>
         <v>000FE670</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="6" t="str">
+      <c r="C49" s="13" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$54)</f>
         <v>bne 0x000FE684</v>
       </c>
-      <c r="D49" s="5"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" t="str">
         <f t="shared" ref="A50" si="37">DEC2HEX(HEX2DEC(A49)+4,8)</f>
         <v>000FE674</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C50" s="4" t="str">
+      <c r="C50" s="8" t="str">
         <f>SUBSTITUTE(C37,"push","pop")</f>
         <v>pop {r4, r5, lr}</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:4">
       <c r="A51" t="str">
         <f t="shared" ref="A51" si="38">DEC2HEX(HEX2DEC(A50)+4,8)</f>
         <v>000FE678</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="8" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:4">
       <c r="A52" t="str">
         <f t="shared" ref="A52" si="39">DEC2HEX(HEX2DEC(A51)+4,8)</f>
         <v>000FE67C</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="8" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:4">
       <c r="A53" t="str">
         <f t="shared" ref="A53" si="40">DEC2HEX(HEX2DEC(A52)+4,8)</f>
         <v>000FE680</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="8" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:4">
       <c r="A54" t="str">
         <f t="shared" ref="A54" si="41">DEC2HEX(HEX2DEC(A53)+4,8)</f>
         <v>000FE684</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C54" s="4" t="str">
+      <c r="C54" s="8" t="str">
         <f>SUBSTITUTE(C50,"lr","pc")</f>
         <v>pop {r4, r5, pc}</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C55" s="1"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A56" s="3" t="s">
+    <row r="55" spans="1:4">
+      <c r="C55" s="10"/>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C56" s="1"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C56" s="10"/>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" t="str">
         <f>DEC2HEX(HEX2DEC(A54)+4,8)</f>
         <v>000FE688</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:4">
       <c r="A58" t="str">
         <f t="shared" ref="A58:A78" si="42">DEC2HEX(HEX2DEC(A57)+4,8)</f>
         <v>000FE68C</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:4">
       <c r="A59" t="str">
         <f t="shared" si="42"/>
         <v>000FE690</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A60" s="7" t="str">
+    <row r="60" spans="1:4">
+      <c r="A60" s="4" t="str">
         <f t="shared" si="42"/>
         <v>000FE694</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="B60" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C60" s="8" t="s">
+      <c r="C60" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D60" s="7" t="s">
+      <c r="D60" s="15" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A61" s="7" t="str">
+    <row r="61" spans="1:4">
+      <c r="A61" s="4" t="str">
         <f t="shared" si="42"/>
         <v>000FE698</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C61" s="8" t="s">
+      <c r="C61" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="D61" s="7"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A62" s="7" t="str">
+      <c r="D61" s="15"/>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="4" t="str">
         <f t="shared" si="42"/>
         <v>000FE69C</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B62" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="C62" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D62" s="7"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A63" s="7" t="str">
+      <c r="D62" s="15"/>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="4" t="str">
         <f t="shared" si="42"/>
         <v>000FE6A0</v>
       </c>
-      <c r="B63" s="7" t="s">
+      <c r="B63" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="8" t="str">
+      <c r="C63" s="14" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$78)</f>
         <v>bne 0x000FE6DC</v>
       </c>
-      <c r="D63" s="7"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A64" s="5" t="str">
+      <c r="D63" s="15"/>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="3" t="str">
         <f t="shared" si="42"/>
         <v>000FE6A4</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D64" s="5" t="s">
+      <c r="D64" s="12" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A65" s="5" t="str">
+    <row r="65" spans="1:4">
+      <c r="A65" s="3" t="str">
         <f t="shared" si="42"/>
         <v>000FE6A8</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C65" s="6" t="s">
+      <c r="C65" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D65" s="5"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A66" s="5" t="str">
+      <c r="D65" s="12"/>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="3" t="str">
         <f t="shared" si="42"/>
         <v>000FE6AC</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="D66" s="5"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A67" s="5" t="str">
+      <c r="D66" s="12"/>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="3" t="str">
         <f t="shared" si="42"/>
         <v>000FE6B0</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="C67" s="6" t="s">
+      <c r="C67" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D67" s="5"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A68" s="5" t="str">
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="3" t="str">
         <f t="shared" si="42"/>
         <v>000FE6B4</v>
       </c>
-      <c r="B68" s="6" t="s">
+      <c r="B68" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C68" s="6" t="s">
+      <c r="C68" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D68" s="5"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A69" s="5" t="str">
+      <c r="D68" s="12"/>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="3" t="str">
         <f t="shared" si="42"/>
         <v>000FE6B8</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C69" s="6" t="str">
+      <c r="C69" s="13" t="str">
         <f>C63</f>
         <v>bne 0x000FE6DC</v>
       </c>
-      <c r="D69" s="5"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A70" s="9" t="str">
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="5" t="str">
         <f t="shared" si="42"/>
         <v>000FE6BC</v>
       </c>
-      <c r="B70" s="9" t="s">
+      <c r="B70" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="C70" s="10" t="s">
+      <c r="C70" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D70" s="9" t="s">
+      <c r="D70" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A71" s="9" t="str">
+    <row r="71" spans="1:4">
+      <c r="A71" s="5" t="str">
         <f t="shared" si="42"/>
         <v>000FE6C0</v>
       </c>
-      <c r="B71" s="9" t="s">
+      <c r="B71" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="C71" s="10" t="s">
+      <c r="C71" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="D71" s="9"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A72" s="9" t="str">
+      <c r="D71" s="16"/>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="5" t="str">
         <f t="shared" si="42"/>
         <v>000FE6C4</v>
       </c>
-      <c r="B72" s="10" t="s">
+      <c r="B72" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="C72" s="10" t="s">
+      <c r="C72" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D72" s="9"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A73" s="9" t="str">
+      <c r="D72" s="16"/>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="5" t="str">
         <f t="shared" si="42"/>
         <v>000FE6C8</v>
       </c>
-      <c r="B73" s="9" t="s">
+      <c r="B73" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="C73" s="10" t="str">
+      <c r="C73" s="17" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$78)</f>
         <v>bne 0x000FE6DC</v>
       </c>
-      <c r="D73" s="9"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D73" s="16"/>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" t="str">
         <f t="shared" si="42"/>
         <v>000FE6CC</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C74" s="4" t="str">
+      <c r="C74" s="8" t="str">
         <f>SUBSTITUTE(C57,"push","pop")</f>
         <v>pop {r4, r5, lr}</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:4">
       <c r="A75" t="str">
         <f t="shared" si="42"/>
         <v>000FE6D0</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="C75" s="8" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:4">
       <c r="A76" t="str">
         <f t="shared" si="42"/>
         <v>000FE6D4</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="C76" s="8" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:4">
       <c r="A77" t="str">
         <f t="shared" si="42"/>
         <v>000FE6D8</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C77" s="8" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:4">
       <c r="A78" t="str">
         <f t="shared" si="42"/>
         <v>000FE6DC</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C78" s="4" t="str">
+      <c r="C78" s="8" t="str">
         <f>SUBSTITUTE(C74,"lr","pc")</f>
         <v>pop {r4, r5, pc}</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="C79" s="1"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A80" s="3" t="s">
+    <row r="79" spans="1:4">
+      <c r="C79" s="10"/>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C80" s="1"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="C80" s="10"/>
+    </row>
+    <row r="81" spans="1:6">
       <c r="A81" t="str">
         <f>DEC2HEX(HEX2DEC(A78)+4,8)</f>
         <v>000FE6E0</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C81" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:6">
       <c r="A82" t="str">
         <f t="shared" ref="A82:A110" si="43">DEC2HEX(HEX2DEC(A81)+4,8)</f>
         <v>000FE6E4</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:6">
       <c r="A83" t="str">
         <f t="shared" si="43"/>
         <v>000FE6E8</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C83" s="4" t="s">
+      <c r="C83" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A84" s="7" t="str">
+    <row r="84" spans="1:6">
+      <c r="A84" s="4" t="str">
         <f t="shared" si="43"/>
         <v>000FE6EC</v>
       </c>
-      <c r="B84" s="7" t="s">
+      <c r="B84" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C84" s="8" t="s">
+      <c r="C84" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D84" s="7" t="s">
+      <c r="D84" s="15" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A85" s="7" t="str">
+    <row r="85" spans="1:6">
+      <c r="A85" s="4" t="str">
         <f t="shared" si="43"/>
         <v>000FE6F0</v>
       </c>
-      <c r="B85" s="7" t="s">
+      <c r="B85" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C85" s="8" t="s">
+      <c r="C85" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="D85" s="7"/>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A86" s="7" t="str">
+      <c r="D85" s="15"/>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" s="4" t="str">
         <f t="shared" si="43"/>
         <v>000FE6F4</v>
       </c>
-      <c r="B86" s="8" t="s">
+      <c r="B86" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C86" s="8" t="s">
+      <c r="C86" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D86" s="7"/>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A87" s="7" t="str">
+      <c r="D86" s="15"/>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="4" t="str">
         <f t="shared" si="43"/>
         <v>000FE6F8</v>
       </c>
-      <c r="B87" s="7" t="s">
+      <c r="B87" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="C87" s="8" t="str">
+      <c r="C87" s="14" t="str">
         <f>_xlfn.CONCAT("beq 0x",A$92)</f>
         <v>beq 0x000FE70C</v>
       </c>
-      <c r="D87" s="7"/>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A88" s="5" t="str">
+      <c r="D87" s="15"/>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="3" t="str">
         <f t="shared" ref="A88" si="44">DEC2HEX(HEX2DEC(A87)+4,8)</f>
         <v>000FE6FC</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B88" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C88" s="6" t="s">
+      <c r="C88" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="D88" s="12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A89" s="5" t="str">
+    <row r="89" spans="1:6">
+      <c r="A89" s="3" t="str">
         <f t="shared" ref="A89" si="45">DEC2HEX(HEX2DEC(A88)+4,8)</f>
         <v>000FE700</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="B89" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="C89" s="6" t="s">
+      <c r="C89" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="D89" s="5"/>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A90" s="5" t="str">
+      <c r="D89" s="12"/>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" s="3" t="str">
         <f t="shared" ref="A90" si="46">DEC2HEX(HEX2DEC(A89)+4,8)</f>
         <v>000FE704</v>
       </c>
-      <c r="B90" s="6" t="s">
+      <c r="B90" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C90" s="6" t="s">
+      <c r="C90" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D90" s="5"/>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A91" s="5" t="str">
+      <c r="D90" s="12"/>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="3" t="str">
         <f t="shared" ref="A91" si="47">DEC2HEX(HEX2DEC(A90)+4,8)</f>
         <v>000FE708</v>
       </c>
-      <c r="B91" s="5" t="s">
+      <c r="B91" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="C91" s="6" t="str">
+      <c r="C91" s="13" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$108)</f>
         <v>bne 0x000FE74C</v>
       </c>
-      <c r="D91" s="5"/>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A92" s="9" t="str">
+      <c r="D91" s="12"/>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE70C</v>
       </c>
-      <c r="B92" s="9" t="s">
+      <c r="B92" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C92" s="10" t="s">
+      <c r="C92" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D92" s="9" t="s">
+      <c r="D92" s="16" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A93" s="9" t="str">
+    <row r="93" spans="1:6">
+      <c r="A93" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE710</v>
       </c>
-      <c r="B93" s="9" t="s">
+      <c r="B93" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="C93" s="10" t="s">
+      <c r="C93" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="D93" s="9"/>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A94" s="9" t="str">
+      <c r="D93" s="16"/>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE714</v>
       </c>
-      <c r="B94" s="10" t="s">
+      <c r="B94" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="C94" s="10" t="s">
+      <c r="C94" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="D94" s="9" t="s">
+      <c r="D94" s="16" t="s">
         <v>188</v>
       </c>
       <c r="E94" t="s">
@@ -2321,18 +2331,18 @@
         <v>20</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A95" s="9" t="str">
+    <row r="95" spans="1:6">
+      <c r="A95" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE718</v>
       </c>
-      <c r="B95" s="9" t="s">
+      <c r="B95" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="C95" s="10" t="s">
+      <c r="C95" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="D95" s="9" t="s">
+      <c r="D95" s="16" t="s">
         <v>190</v>
       </c>
       <c r="E95" t="s">
@@ -2342,195 +2352,195 @@
         <v>27</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A96" s="9" t="str">
+    <row r="96" spans="1:6">
+      <c r="A96" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE71C</v>
       </c>
-      <c r="B96" s="9" t="s">
+      <c r="B96" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="C96" s="10" t="str">
+      <c r="C96" s="17" t="str">
         <f>_xlfn.CONCAT("beq 0x",A100)</f>
         <v>beq 0x000FE72C</v>
       </c>
-      <c r="D96" s="9"/>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A97" s="9" t="str">
+      <c r="D96" s="16"/>
+    </row>
+    <row r="97" spans="1:7">
+      <c r="A97" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE720</v>
       </c>
-      <c r="B97" s="9" t="s">
+      <c r="B97" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="C97" s="10" t="s">
+      <c r="C97" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="D97" s="16" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A98" s="9" t="str">
+    <row r="98" spans="1:7">
+      <c r="A98" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE724</v>
       </c>
-      <c r="B98" s="9" t="s">
+      <c r="B98" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="C98" s="10" t="str">
+      <c r="C98" s="17" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$108)</f>
         <v>bne 0x000FE74C</v>
       </c>
-      <c r="D98" s="9"/>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A99" s="9" t="str">
+      <c r="D98" s="16"/>
+    </row>
+    <row r="99" spans="1:7">
+      <c r="A99" s="5" t="str">
         <f t="shared" si="43"/>
         <v>000FE728</v>
       </c>
-      <c r="B99" s="9" t="s">
+      <c r="B99" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="C99" s="10" t="s">
+      <c r="C99" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="D99" s="16" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:7">
       <c r="A100" t="str">
         <f t="shared" si="43"/>
         <v>000FE72C</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="C100" s="4" t="str">
+      <c r="C100" s="8" t="str">
         <f>_xlfn.CONCAT("ldr r7, [pc, 0x",DEC2HEX(HEX2DEC(A110)-HEX2DEC(A100)-8,3),"]")</f>
         <v>ldr r7, [pc, 0x020]</v>
       </c>
-      <c r="D100" t="s">
+      <c r="D100" s="9" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:7">
       <c r="A101" t="str">
         <f t="shared" si="43"/>
         <v>000FE730</v>
       </c>
-      <c r="B101" s="4" t="s">
+      <c r="B101" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C101" s="4" t="s">
+      <c r="C101" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D101" t="s">
+      <c r="D101" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:7">
       <c r="A102" t="str">
         <f t="shared" si="43"/>
         <v>000FE734</v>
       </c>
-      <c r="B102" s="4" t="s">
+      <c r="B102" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C102" s="4" t="s">
+      <c r="C102" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D102" t="s">
+      <c r="D102" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:7">
       <c r="A103" t="str">
         <f t="shared" si="43"/>
         <v>000FE738</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C103" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D103" t="s">
+      <c r="D103" s="9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:7">
       <c r="A104" t="str">
         <f t="shared" si="43"/>
         <v>000FE73C</v>
       </c>
-      <c r="B104" s="4" t="s">
+      <c r="B104" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="C104" s="4" t="s">
+      <c r="C104" s="8" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:7">
       <c r="A105" t="str">
         <f t="shared" si="43"/>
         <v>000FE740</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C105" s="4" t="str">
+      <c r="C105" s="8" t="str">
         <f>_xlfn.CONCAT("bhs 0x",A$108)</f>
         <v>bhs 0x000FE74C</v>
       </c>
-      <c r="D105" t="s">
+      <c r="D105" s="9" t="s">
         <v>172</v>
       </c>
       <c r="F105" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:7">
       <c r="A106" t="str">
         <f t="shared" si="43"/>
         <v>000FE744</v>
       </c>
-      <c r="B106" s="4" t="s">
+      <c r="B106" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C106" s="4" t="s">
+      <c r="C106" s="8" t="s">
         <v>70</v>
       </c>
       <c r="F106" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:7">
       <c r="A107" t="str">
         <f t="shared" si="43"/>
         <v>000FE748</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="C107" t="s">
+      <c r="C107" s="9" t="s">
         <v>96</v>
       </c>
       <c r="F107" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:7">
       <c r="A108" t="str">
         <f t="shared" si="43"/>
         <v>000FE74C</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C108" s="4" t="str">
+      <c r="C108" s="8" t="str">
         <f>SUBSTITUTE(C81,"push","pop")</f>
         <v>pop {r4, r5, r6, r7, lr}</v>
       </c>
@@ -2538,30 +2548,30 @@
         <v>66</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:7">
       <c r="A109" t="str">
         <f t="shared" si="43"/>
         <v>000FE750</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C109" s="4" t="s">
+      <c r="C109" s="8" t="s">
         <v>34</v>
       </c>
       <c r="F109" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:7">
       <c r="A110" t="str">
         <f t="shared" si="43"/>
         <v>000FE754</v>
       </c>
-      <c r="B110" s="4" t="s">
+      <c r="B110" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C110" t="s">
+      <c r="C110" s="9" t="s">
         <v>36</v>
       </c>
       <c r="F110" t="s">
@@ -2572,500 +2582,500 @@
         <v>Apex Bulbasaur, Electivire, Magmortar, Heatran, Rotom-H, Mega Togedemaru</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="C112" s="1"/>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A113" s="3" t="s">
+    <row r="112" spans="1:7">
+      <c r="C112" s="10"/>
+    </row>
+    <row r="113" spans="1:5">
+      <c r="A113" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C113" s="1"/>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="C113" s="10"/>
+    </row>
+    <row r="114" spans="1:5">
       <c r="A114" t="str">
         <f>DEC2HEX(HEX2DEC(A110)+4,8)</f>
         <v>000FE758</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="C114" t="s">
+      <c r="C114" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:5">
       <c r="A115" t="str">
         <f t="shared" ref="A115:A148" si="48">DEC2HEX(HEX2DEC(A114)+4,8)</f>
         <v>000FE75C</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C115" t="s">
+      <c r="C115" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:5">
       <c r="A116" t="str">
         <f t="shared" si="48"/>
         <v>000FE760</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C116" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A117" s="7" t="str">
+    <row r="117" spans="1:5">
+      <c r="A117" s="4" t="str">
         <f t="shared" si="48"/>
         <v>000FE764</v>
       </c>
-      <c r="B117" s="7" t="s">
+      <c r="B117" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C117" s="8" t="s">
+      <c r="C117" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D117" s="7" t="s">
+      <c r="D117" s="15" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A118" s="7" t="str">
+    <row r="118" spans="1:5">
+      <c r="A118" s="4" t="str">
         <f t="shared" si="48"/>
         <v>000FE768</v>
       </c>
-      <c r="B118" s="7" t="s">
+      <c r="B118" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="C118" s="8" t="s">
+      <c r="C118" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="D118" s="7"/>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A119" s="7" t="str">
+      <c r="D118" s="15"/>
+    </row>
+    <row r="119" spans="1:5">
+      <c r="A119" s="4" t="str">
         <f t="shared" si="48"/>
         <v>000FE76C</v>
       </c>
-      <c r="B119" s="8" t="s">
+      <c r="B119" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C119" s="8" t="s">
+      <c r="C119" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D119" s="7"/>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A120" s="7" t="str">
+      <c r="D119" s="15"/>
+    </row>
+    <row r="120" spans="1:5">
+      <c r="A120" s="4" t="str">
         <f t="shared" si="48"/>
         <v>000FE770</v>
       </c>
-      <c r="B120" s="7" t="s">
+      <c r="B120" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="C120" s="8" t="str">
+      <c r="C120" s="14" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$147)</f>
         <v>bne 0x000FE7DC</v>
       </c>
-      <c r="D120" s="7"/>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A121" s="5" t="str">
+      <c r="D120" s="15"/>
+    </row>
+    <row r="121" spans="1:5">
+      <c r="A121" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE774</v>
       </c>
-      <c r="B121" s="5" t="s">
+      <c r="B121" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C121" s="6" t="s">
+      <c r="C121" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D121" s="5" t="s">
+      <c r="D121" s="12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A122" s="5" t="str">
+    <row r="122" spans="1:5">
+      <c r="A122" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE778</v>
       </c>
-      <c r="B122" s="5" t="s">
+      <c r="B122" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="C122" s="6" t="s">
+      <c r="C122" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="D122" s="5"/>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A123" s="5" t="str">
+      <c r="D122" s="12"/>
+    </row>
+    <row r="123" spans="1:5">
+      <c r="A123" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE77C</v>
       </c>
-      <c r="B123" s="6" t="s">
+      <c r="B123" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="C123" s="6" t="s">
+      <c r="C123" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D123" s="5" t="s">
+      <c r="D123" s="12" t="s">
         <v>192</v>
       </c>
       <c r="E123" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A124" s="5" t="str">
+    <row r="124" spans="1:5">
+      <c r="A124" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE780</v>
       </c>
-      <c r="B124" s="5" t="s">
+      <c r="B124" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="C124" s="6" t="s">
+      <c r="C124" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="D124" s="5" t="s">
+      <c r="D124" s="12" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A125" s="5" t="str">
+    <row r="125" spans="1:5">
+      <c r="A125" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE784</v>
       </c>
-      <c r="B125" s="5" t="s">
+      <c r="B125" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="C125" s="6" t="str">
+      <c r="C125" s="13" t="str">
         <f>_xlfn.CONCAT("beq 0x",A129)</f>
         <v>beq 0x000FE794</v>
       </c>
-      <c r="D125" s="5"/>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A126" s="5" t="str">
+      <c r="D125" s="12"/>
+    </row>
+    <row r="126" spans="1:5">
+      <c r="A126" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE788</v>
       </c>
-      <c r="B126" s="5" t="s">
+      <c r="B126" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="C126" s="6" t="s">
+      <c r="C126" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D126" s="5" t="s">
+      <c r="D126" s="12" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A127" s="5" t="str">
+    <row r="127" spans="1:5">
+      <c r="A127" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE78C</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="B127" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="C127" s="6" t="str">
+      <c r="C127" s="13" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$147)</f>
         <v>bne 0x000FE7DC</v>
       </c>
-      <c r="D127" s="5"/>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A128" s="5" t="str">
+      <c r="D127" s="12"/>
+    </row>
+    <row r="128" spans="1:5">
+      <c r="A128" s="3" t="str">
         <f t="shared" si="48"/>
         <v>000FE790</v>
       </c>
-      <c r="B128" s="5" t="s">
+      <c r="B128" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="C128" s="6" t="s">
+      <c r="C128" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="D128" s="5" t="s">
+      <c r="D128" s="12" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A129" s="9" t="str">
+    <row r="129" spans="1:4">
+      <c r="A129" s="5" t="str">
         <f t="shared" si="48"/>
         <v>000FE794</v>
       </c>
-      <c r="B129" s="9" t="s">
+      <c r="B129" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="C129" s="10" t="str">
+      <c r="C129" s="17" t="str">
         <f>_xlfn.CONCAT("ldr r7, [pc, 0x",DEC2HEX(HEX2DEC(A148)-HEX2DEC(A129)-8,3),"]")</f>
         <v>ldr r7, [pc, 0x044]</v>
       </c>
-      <c r="D129" s="9" t="s">
+      <c r="D129" s="16" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A130" s="9" t="str">
+    <row r="130" spans="1:4">
+      <c r="A130" s="5" t="str">
         <f t="shared" si="48"/>
         <v>000FE798</v>
       </c>
-      <c r="B130" s="10" t="s">
+      <c r="B130" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="C130" s="10" t="s">
+      <c r="C130" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="D130" s="9" t="s">
+      <c r="D130" s="16" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A131" s="9" t="str">
+    <row r="131" spans="1:4">
+      <c r="A131" s="5" t="str">
         <f t="shared" si="48"/>
         <v>000FE79C</v>
       </c>
-      <c r="B131" s="10" t="s">
+      <c r="B131" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="C131" s="10" t="s">
+      <c r="C131" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="D131" s="9" t="s">
+      <c r="D131" s="16" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A132" s="9" t="str">
+    <row r="132" spans="1:4">
+      <c r="A132" s="5" t="str">
         <f t="shared" si="48"/>
         <v>000FE7A0</v>
       </c>
-      <c r="B132" s="9" t="s">
+      <c r="B132" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="C132" s="10" t="s">
+      <c r="C132" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="D132" s="9" t="s">
+      <c r="D132" s="16" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A133" s="11" t="str">
+    <row r="133" spans="1:4">
+      <c r="A133" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7A4</v>
       </c>
-      <c r="B133" s="11" t="s">
+      <c r="B133" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="C133" s="11" t="s">
+      <c r="C133" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D133" s="11" t="s">
+      <c r="D133" s="19" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A134" s="11" t="str">
+    <row r="134" spans="1:4">
+      <c r="A134" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7A8</v>
       </c>
-      <c r="B134" s="11" t="s">
+      <c r="B134" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="C134" s="11" t="s">
+      <c r="C134" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D134" s="11"/>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A135" s="11" t="str">
+      <c r="D134" s="19"/>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7AC</v>
       </c>
-      <c r="B135" s="11" t="s">
+      <c r="B135" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="C135" s="11" t="s">
+      <c r="C135" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="D135" s="11"/>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A136" s="11" t="str">
+      <c r="D135" s="19"/>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7B0</v>
       </c>
-      <c r="B136" s="11" t="s">
+      <c r="B136" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="C136" s="11" t="s">
+      <c r="C136" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="D136" s="11"/>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A137" s="11" t="str">
+      <c r="D136" s="19"/>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7B4</v>
       </c>
-      <c r="B137" s="12" t="s">
+      <c r="B137" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="C137" s="11" t="s">
+      <c r="C137" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="D137" s="11" t="s">
+      <c r="D137" s="19" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A138" s="11" t="str">
+    <row r="138" spans="1:4">
+      <c r="A138" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7B8</v>
       </c>
-      <c r="B138" s="12" t="s">
+      <c r="B138" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="C138" s="11" t="s">
+      <c r="C138" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D138" s="11" t="s">
+      <c r="D138" s="19" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A139" s="11" t="str">
+    <row r="139" spans="1:4">
+      <c r="A139" s="6" t="str">
         <f t="shared" si="48"/>
         <v>000FE7BC</v>
       </c>
-      <c r="B139" s="12" t="s">
+      <c r="B139" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="C139" s="11" t="s">
+      <c r="C139" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="D139" s="11"/>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D139" s="19"/>
+    </row>
+    <row r="140" spans="1:4">
       <c r="A140" t="str">
         <f t="shared" si="48"/>
         <v>000FE7C0</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="C140" s="4" t="s">
+      <c r="C140" s="8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:4">
       <c r="A141" t="str">
         <f t="shared" si="48"/>
         <v>000FE7C4</v>
       </c>
-      <c r="B141" s="4" t="s">
+      <c r="B141" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C141" s="4" t="s">
+      <c r="C141" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D141" t="s">
+      <c r="D141" s="9" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:4">
       <c r="A142" t="str">
         <f t="shared" si="48"/>
         <v>000FE7C8</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B142" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C142" s="4" t="s">
+      <c r="C142" s="8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:4">
       <c r="A143" t="str">
         <f t="shared" si="48"/>
         <v>000FE7CC</v>
       </c>
-      <c r="B143" s="4" t="s">
+      <c r="B143" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C143" s="4" t="s">
+      <c r="C143" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D143" t="s">
+      <c r="D143" s="9" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:4">
       <c r="A144" t="str">
         <f t="shared" si="48"/>
         <v>000FE7D0</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B144" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C144" s="4" t="str">
+      <c r="C144" s="8" t="str">
         <f>SUBSTITUTE(C114,"push","pop")</f>
         <v>pop {r4, r5, r6, r7, lr}</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:9">
       <c r="A145" t="str">
         <f t="shared" si="48"/>
         <v>000FE7D4</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B145" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="C145" t="s">
+      <c r="C145" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:9">
       <c r="A146" t="str">
         <f t="shared" si="48"/>
         <v>000FE7D8</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B146" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="C146" s="4" t="s">
+      <c r="C146" s="8" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:9">
       <c r="A147" t="str">
         <f t="shared" si="48"/>
         <v>000FE7DC</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B147" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C147" t="str">
+      <c r="C147" s="9" t="str">
         <f>SUBSTITUTE(C144,"lr","pc")</f>
         <v>pop {r4, r5, r6, r7, pc}</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:9">
       <c r="A148" t="str">
         <f t="shared" si="48"/>
         <v>000FE7E0</v>
       </c>
-      <c r="B148" s="4" t="s">
+      <c r="B148" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C148" t="s">
+      <c r="C148" s="9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:9">
       <c r="F149">
         <v>0</v>
       </c>
@@ -3080,7 +3090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:9">
       <c r="F150">
         <v>1</v>
       </c>
@@ -3097,7 +3107,7 @@
         <v>1.03125</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:9">
       <c r="F151">
         <f>F150+1</f>
         <v>2</v>
@@ -3115,7 +3125,7 @@
         <v>1.0625</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:9">
       <c r="F152">
         <f t="shared" ref="F152:F164" si="51">F151+1</f>
         <v>3</v>
@@ -3133,7 +3143,7 @@
         <v>1.09375</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:9">
       <c r="F153">
         <f t="shared" si="51"/>
         <v>4</v>
@@ -3151,7 +3161,7 @@
         <v>1.125</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:9">
       <c r="F154">
         <f t="shared" si="51"/>
         <v>5</v>
@@ -3169,7 +3179,7 @@
         <v>1.15625</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:9">
       <c r="F155">
         <f t="shared" si="51"/>
         <v>6</v>
@@ -3187,7 +3197,7 @@
         <v>1.1875</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:9">
       <c r="F156">
         <f t="shared" si="51"/>
         <v>7</v>
@@ -3205,7 +3215,7 @@
         <v>1.21875</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:9">
       <c r="F157">
         <f t="shared" si="51"/>
         <v>8</v>
@@ -3223,7 +3233,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:9">
       <c r="F158">
         <f t="shared" si="51"/>
         <v>9</v>
@@ -3241,7 +3251,7 @@
         <v>1.28125</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:9">
       <c r="F159">
         <f t="shared" si="51"/>
         <v>10</v>
@@ -3259,7 +3269,7 @@
         <v>1.3125</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:9">
       <c r="F160">
         <f t="shared" si="51"/>
         <v>11</v>
@@ -3277,7 +3287,7 @@
         <v>1.34375</v>
       </c>
     </row>
-    <row r="161" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="161" spans="6:9">
       <c r="F161">
         <f t="shared" si="51"/>
         <v>12</v>
@@ -3295,7 +3305,7 @@
         <v>1.375</v>
       </c>
     </row>
-    <row r="162" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="162" spans="6:9">
       <c r="F162">
         <f t="shared" si="51"/>
         <v>13</v>
@@ -3313,7 +3323,7 @@
         <v>1.40625</v>
       </c>
     </row>
-    <row r="163" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="163" spans="6:9">
       <c r="F163">
         <f t="shared" si="51"/>
         <v>14</v>
@@ -3331,7 +3341,7 @@
         <v>1.4375</v>
       </c>
     </row>
-    <row r="164" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="164" spans="6:9">
       <c r="F164">
         <f t="shared" si="51"/>
         <v>15</v>
@@ -3349,7 +3359,7 @@
         <v>1.46875</v>
       </c>
     </row>
-    <row r="165" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="165" spans="6:9">
       <c r="F165">
         <f>F164+1</f>
         <v>16</v>
@@ -3367,7 +3377,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="166" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="166" spans="6:9">
       <c r="F166">
         <f t="shared" ref="F166:F172" si="53">F165+1</f>
         <v>17</v>
@@ -3385,7 +3395,7 @@
         <v>1.53125</v>
       </c>
     </row>
-    <row r="167" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="167" spans="6:9">
       <c r="F167">
         <f t="shared" si="53"/>
         <v>18</v>
@@ -3403,7 +3413,7 @@
         <v>1.5625</v>
       </c>
     </row>
-    <row r="168" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="168" spans="6:9">
       <c r="F168">
         <f t="shared" si="53"/>
         <v>19</v>
@@ -3421,7 +3431,7 @@
         <v>1.59375</v>
       </c>
     </row>
-    <row r="169" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="169" spans="6:9">
       <c r="F169">
         <f t="shared" si="53"/>
         <v>20</v>
@@ -3439,7 +3449,7 @@
         <v>1.625</v>
       </c>
     </row>
-    <row r="170" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="170" spans="6:9">
       <c r="F170">
         <f t="shared" si="53"/>
         <v>21</v>
@@ -3457,7 +3467,7 @@
         <v>1.65625</v>
       </c>
     </row>
-    <row r="171" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="171" spans="6:9">
       <c r="F171">
         <f t="shared" si="53"/>
         <v>22</v>
@@ -3475,7 +3485,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="172" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="172" spans="6:9">
       <c r="F172">
         <f t="shared" si="53"/>
         <v>23</v>
@@ -3493,7 +3503,7 @@
         <v>1.71875</v>
       </c>
     </row>
-    <row r="173" spans="6:9" x14ac:dyDescent="0.45">
+    <row r="173" spans="6:9">
       <c r="F173">
         <f>F172+1</f>
         <v>24</v>
@@ -3520,12 +3530,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C67D84D5-4D25-4A23-9C85-7AF2BA13284F}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.15"/>
   <cols>
-    <col min="1" max="1" width="53.9296875" customWidth="1"/>
+    <col min="1" max="1" width="53.92578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>83</v>
       </c>
@@ -3534,7 +3544,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
Refactor USUM patch engine, fix 64-bit Citra load truncation, clean repository and build setup
</commit_message>
<xml_diff>
--- a/ARM Functions/Ability Edits/Electropyresis.xlsx
+++ b/ARM Functions/Ability Edits/Electropyresis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\ROM\3ds\USUM ARM research\Ability Edits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FFBA8F-9D65-490A-8D20-4B041D5E95A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B546DCDB-13E7-4E4E-B5CB-64A46E437B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16457" yWindow="0" windowWidth="16457" windowHeight="17914" xr2:uid="{DFD0B34E-FAAD-4BE6-8FC0-3053B30C3017}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" xr2:uid="{DFD0B34E-FAAD-4BE6-8FC0-3053B30C3017}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="215">
   <si>
     <t>mov r1, r4</t>
   </si>
@@ -183,9 +183,6 @@
     <t>get current Type</t>
   </si>
   <si>
-    <t>Don't modify Ground immune electric</t>
-  </si>
-  <si>
     <t>mov r0, 0x3D</t>
   </si>
   <si>
@@ -342,21 +339,9 @@
     <t>0400A0E3</t>
   </si>
   <si>
-    <t>5925FEEB</t>
-  </si>
-  <si>
-    <t>1000001A</t>
-  </si>
-  <si>
-    <t>5525FEEB</t>
-  </si>
-  <si>
     <t>0040A0E1</t>
   </si>
   <si>
-    <t>5225FEEB</t>
-  </si>
-  <si>
     <t>040050E3</t>
   </si>
   <si>
@@ -594,9 +579,6 @@
     <t>1800A0E3</t>
   </si>
   <si>
-    <t>0800000A</t>
-  </si>
-  <si>
     <t>Defensive 0x4E/0x4F</t>
   </si>
   <si>
@@ -630,15 +612,6 @@
     <t xml:space="preserve">bl 0x00087B58 </t>
   </si>
   <si>
-    <t>cmpeq r4, 0xC</t>
-  </si>
-  <si>
-    <t>Defending is Ground</t>
-  </si>
-  <si>
-    <t>Offending is Electric</t>
-  </si>
-  <si>
     <t>cmp r4, 0x6</t>
   </si>
   <si>
@@ -654,15 +627,6 @@
     <t>Offending Type not in list</t>
   </si>
   <si>
-    <t>nop</t>
-  </si>
-  <si>
-    <t>00F020E3</t>
-  </si>
-  <si>
-    <t>0C005403</t>
-  </si>
-  <si>
     <t>060054E3</t>
   </si>
   <si>
@@ -682,22 +646,50 @@
   </si>
   <si>
     <t>0x80*(value loaded + conditional 0xC) is %</t>
+  </si>
+  <si>
+    <t>bl 0x000FDEB8</t>
+  </si>
+  <si>
+    <t>get multiplier</t>
+  </si>
+  <si>
+    <t>cmp r0, 0x7</t>
+  </si>
+  <si>
+    <t>070050E3</t>
+  </si>
+  <si>
+    <t>mov r1, 0x5</t>
+  </si>
+  <si>
+    <t>5A25FEEB</t>
+  </si>
+  <si>
+    <t>1100001A</t>
+  </si>
+  <si>
+    <t>5625FEEB</t>
+  </si>
+  <si>
+    <t>4E25FEEB</t>
+  </si>
+  <si>
+    <t>24FEFFEB</t>
+  </si>
+  <si>
+    <t>0300009A</t>
+  </si>
+  <si>
+    <t>0510A0E3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -723,7 +715,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -754,6 +746,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -767,27 +765,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1125,23 +1121,26 @@
   <dimension ref="A1:O173"/>
   <sheetFormatPr defaultRowHeight="15.9"/>
   <cols>
-    <col min="2" max="2" width="9.35546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="50.78515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.85546875" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3"/>
+    <col min="2" max="2" width="9.35546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.78515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="9.140625" style="3"/>
+    <col min="9" max="9" width="16.85546875" style="3" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1149,2375 +1148,2372 @@
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2"/>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C3" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>168</v>
+      <c r="D3" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:15">
-      <c r="A4" t="str">
+      <c r="A4" s="3" t="str">
         <f t="shared" ref="A4:A7" si="0">DEC2HEX(HEX2DEC(A3)+4,8)</f>
         <v>000FE5CC</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:15">
-      <c r="A5" t="str">
+      <c r="A5" s="3" t="str">
         <f t="shared" si="0"/>
         <v>000FE5D0</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:15">
-      <c r="A6" t="str">
+      <c r="A6" s="3" t="str">
         <f t="shared" si="0"/>
         <v>000FE5D4</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:15">
-      <c r="A7" t="str">
+      <c r="A7" s="3" t="str">
         <f t="shared" si="0"/>
         <v>000FE5D8</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:15">
-      <c r="C8" s="10"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="11"/>
+        <v>180</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" t="str">
+      <c r="A10" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(A7)+4,8)</f>
         <v>000FE5DC</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" s="9" t="s">
+      <c r="B10" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:15">
-      <c r="A11" t="str">
-        <f t="shared" ref="A11" si="1">DEC2HEX(HEX2DEC(A10)+4,8)</f>
+      <c r="A11" s="3" t="str">
+        <f t="shared" ref="A11:A12" si="1">DEC2HEX(HEX2DEC(A10)+4,8)</f>
         <v>000FE5E0</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F11" s="2"/>
       <c r="O11" s="2"/>
     </row>
     <row r="12" spans="1:15">
-      <c r="A12" t="str">
-        <f t="shared" ref="A12" si="2">DEC2HEX(HEX2DEC(A11)+4,8)</f>
+      <c r="A12" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>000FE5E4</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>205</v>
-      </c>
+      <c r="B12" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:15">
-      <c r="A13" s="3" t="str">
-        <f t="shared" ref="A13" si="3">DEC2HEX(HEX2DEC(A12)+4,8)</f>
+      <c r="A13" s="6" t="str">
+        <f t="shared" ref="A13" si="2">DEC2HEX(HEX2DEC(A12)+4,8)</f>
         <v>000FE5E8</v>
       </c>
-      <c r="B13" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>42</v>
-      </c>
+      <c r="B13" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D13" s="6"/>
       <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:15">
-      <c r="A14" s="3" t="str">
-        <f t="shared" ref="A14" si="4">DEC2HEX(HEX2DEC(A13)+4,8)</f>
+      <c r="A14" s="6" t="str">
+        <f t="shared" ref="A14" si="3">DEC2HEX(HEX2DEC(A13)+4,8)</f>
         <v>000FE5EC</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="D14" s="12"/>
+      <c r="B14" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="6"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:15">
-      <c r="A15" s="3" t="str">
-        <f t="shared" ref="A15" si="5">DEC2HEX(HEX2DEC(A14)+4,8)</f>
+      <c r="A15" s="6" t="str">
+        <f t="shared" ref="A15" si="4">DEC2HEX(HEX2DEC(A14)+4,8)</f>
         <v>000FE5F0</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="12"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:15">
-      <c r="A16" s="3" t="str">
-        <f t="shared" ref="A16" si="6">DEC2HEX(HEX2DEC(A15)+4,8)</f>
-        <v>000FE5F4</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C16" s="12" t="str">
+      <c r="B15" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C15" s="6" t="str">
         <f>_xlfn.CONCAT("bne 0x",A34)</f>
         <v>bne 0x000FE63C</v>
       </c>
-      <c r="D16" s="12"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" s="9" t="str">
+        <f t="shared" ref="A16" si="5">DEC2HEX(HEX2DEC(A15)+4,8)</f>
+        <v>000FE5F4</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="4" t="str">
-        <f t="shared" ref="A17" si="7">DEC2HEX(HEX2DEC(A16)+4,8)</f>
+      <c r="A17" s="9" t="str">
+        <f t="shared" ref="A17" si="6">DEC2HEX(HEX2DEC(A16)+4,8)</f>
         <v>000FE5F8</v>
       </c>
-      <c r="B17" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>40</v>
-      </c>
+      <c r="B17" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D17" s="9"/>
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="4" t="str">
-        <f t="shared" ref="A18" si="8">DEC2HEX(HEX2DEC(A17)+4,8)</f>
+      <c r="A18" s="9" t="str">
+        <f t="shared" ref="A18:A23" si="7">DEC2HEX(HEX2DEC(A17)+4,8)</f>
         <v>000FE5FC</v>
       </c>
-      <c r="B18" s="15" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="D18" s="15"/>
-      <c r="F18" s="2"/>
+      <c r="B18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="9"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="4" t="str">
-        <f t="shared" ref="A19" si="9">DEC2HEX(HEX2DEC(A18)+4,8)</f>
+      <c r="A19" s="13" t="str">
+        <f t="shared" si="7"/>
         <v>000FE600</v>
       </c>
-      <c r="B19" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="D19" s="15"/>
+      <c r="B19" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="5" t="str">
-        <f t="shared" ref="A20" si="10">DEC2HEX(HEX2DEC(A19)+4,8)</f>
+      <c r="A20" s="13" t="str">
+        <f t="shared" si="7"/>
         <v>000FE604</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>48</v>
-      </c>
+      <c r="B20" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="2"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="5" t="str">
-        <f t="shared" ref="A21" si="11">DEC2HEX(HEX2DEC(A20)+4,8)</f>
+      <c r="A21" s="13" t="str">
+        <f t="shared" si="7"/>
         <v>000FE608</v>
       </c>
-      <c r="B21" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="D21" s="16" t="s">
+      <c r="B21" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="13" t="str">
+        <f t="shared" si="7"/>
+        <v>000FE60C</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="13" t="str">
+        <f t="shared" si="7"/>
+        <v>000FE610</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" s="13" t="str">
+        <f>_xlfn.CONCAT("bne 0x",A$34)</f>
+        <v>bne 0x000FE63C</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="16" t="str">
+        <f t="shared" ref="A24" si="8">DEC2HEX(HEX2DEC(A23)+4,8)</f>
+        <v>000FE614</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="5" t="str">
-        <f t="shared" ref="A22" si="12">DEC2HEX(HEX2DEC(A21)+4,8)</f>
-        <v>000FE60C</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="5" t="str">
-        <f t="shared" ref="A23" si="13">DEC2HEX(HEX2DEC(A22)+4,8)</f>
-        <v>000FE610</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="5" t="str">
-        <f t="shared" ref="A24" si="14">DEC2HEX(HEX2DEC(A23)+4,8)</f>
-        <v>000FE614</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>185</v>
-      </c>
-      <c r="C24" s="16" t="str">
-        <f>_xlfn.CONCAT("beq 0x",A$34)</f>
-        <v>beq 0x000FE63C</v>
-      </c>
-      <c r="D24" s="16"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="6" t="str">
-        <f t="shared" ref="A25" si="15">DEC2HEX(HEX2DEC(A24)+4,8)</f>
+      <c r="A25" s="16" t="str">
+        <f t="shared" ref="A25" si="9">DEC2HEX(HEX2DEC(A24)+4,8)</f>
         <v>000FE618</v>
       </c>
-      <c r="B25" s="18" t="s">
-        <v>208</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
+      <c r="B25" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="D25" s="16"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="6" t="str">
-        <f t="shared" ref="A26" si="16">DEC2HEX(HEX2DEC(A25)+4,8)</f>
+      <c r="A26" s="15" t="str">
+        <f t="shared" ref="A26" si="10">DEC2HEX(HEX2DEC(A25)+4,8)</f>
         <v>000FE61C</v>
       </c>
-      <c r="B26" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>27</v>
+      <c r="B26" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="6" t="str">
-        <f t="shared" ref="A27" si="17">DEC2HEX(HEX2DEC(A26)+4,8)</f>
+      <c r="A27" s="15" t="str">
+        <f t="shared" ref="A27" si="11">DEC2HEX(HEX2DEC(A26)+4,8)</f>
         <v>000FE620</v>
       </c>
-      <c r="B27" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>202</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>20</v>
-      </c>
+      <c r="B27" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="D27" s="15"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="6" t="str">
-        <f t="shared" ref="A28" si="18">DEC2HEX(HEX2DEC(A27)+4,8)</f>
+      <c r="A28" s="15" t="str">
+        <f t="shared" ref="A28:A30" si="12">DEC2HEX(HEX2DEC(A27)+4,8)</f>
         <v>000FE624</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>211</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="D28" s="19" t="s">
-        <v>25</v>
-      </c>
+      <c r="B28" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="D28" s="15"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="6" t="str">
-        <f t="shared" ref="A29" si="19">DEC2HEX(HEX2DEC(A28)+4,8)</f>
+      <c r="A29" s="15" t="str">
+        <f t="shared" si="12"/>
         <v>000FE628</v>
       </c>
-      <c r="B29" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="C29" s="19" t="str">
-        <f>_xlfn.CONCAT("bne 0x",A$34)</f>
-        <v>bne 0x000FE63C</v>
-      </c>
-      <c r="D29" s="19" t="s">
-        <v>204</v>
-      </c>
+      <c r="B29" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="C29" s="15" t="str">
+        <f>_xlfn.CONCAT("bls 0x",A34)</f>
+        <v>bls 0x000FE63C</v>
+      </c>
+      <c r="D29" s="15"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" t="str">
-        <f t="shared" ref="A30" si="20">DEC2HEX(HEX2DEC(A29)+4,8)</f>
+      <c r="A30" s="15" t="str">
+        <f t="shared" si="12"/>
         <v>000FE62C</v>
       </c>
-      <c r="B30" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>46</v>
+      <c r="B30" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" t="str">
-        <f t="shared" ref="A31" si="21">DEC2HEX(HEX2DEC(A30)+4,8)</f>
+      <c r="A31" s="3" t="str">
+        <f t="shared" ref="A31" si="13">DEC2HEX(HEX2DEC(A30)+4,8)</f>
         <v>000FE630</v>
       </c>
-      <c r="B31" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>49</v>
+      <c r="B31" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" t="str">
-        <f t="shared" ref="A32" si="22">DEC2HEX(HEX2DEC(A31)+4,8)</f>
+      <c r="A32" s="3" t="str">
+        <f t="shared" ref="A32" si="14">DEC2HEX(HEX2DEC(A31)+4,8)</f>
         <v>000FE634</v>
       </c>
-      <c r="B32" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="C32" s="8" t="str">
+      <c r="B32" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="3" t="str">
         <f>SUBSTITUTE(C10,"push","pop")</f>
         <v>pop {r4, lr}</v>
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" t="str">
-        <f t="shared" ref="A33" si="23">DEC2HEX(HEX2DEC(A32)+4,8)</f>
+      <c r="A33" s="3" t="str">
+        <f t="shared" ref="A33" si="15">DEC2HEX(HEX2DEC(A32)+4,8)</f>
         <v>000FE638</v>
       </c>
-      <c r="B33" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="C33" s="9" t="s">
+      <c r="B33" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" t="str">
-        <f t="shared" ref="A34" si="24">DEC2HEX(HEX2DEC(A33)+4,8)</f>
+      <c r="A34" s="3" t="str">
+        <f t="shared" ref="A34" si="16">DEC2HEX(HEX2DEC(A33)+4,8)</f>
         <v>000FE63C</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="C34" s="8" t="str">
-        <f>SUBSTITUTE(C32,"lr","pc")</f>
+      <c r="B34" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="2" t="str">
+        <f>SUBSTITUTE(SUBSTITUTE(C10,"push","pop"),"lr","pc")</f>
         <v>pop {r4, pc}</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="C35" s="10"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C36" s="10"/>
+        <v>49</v>
+      </c>
+      <c r="C36" s="4"/>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" t="str">
+      <c r="A37" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(A34)+4,8)</f>
         <v>000FE640</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" t="str">
-        <f t="shared" ref="A38" si="25">DEC2HEX(HEX2DEC(A37)+4,8)</f>
+      <c r="A38" s="3" t="str">
+        <f t="shared" ref="A38" si="17">DEC2HEX(HEX2DEC(A37)+4,8)</f>
         <v>000FE644</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" t="str">
-        <f t="shared" ref="A39" si="26">DEC2HEX(HEX2DEC(A38)+4,8)</f>
+      <c r="A39" s="3" t="str">
+        <f t="shared" ref="A39" si="18">DEC2HEX(HEX2DEC(A38)+4,8)</f>
         <v>000FE648</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="4" t="str">
-        <f t="shared" ref="A40" si="27">DEC2HEX(HEX2DEC(A39)+4,8)</f>
+      <c r="A40" s="9" t="str">
+        <f t="shared" ref="A40" si="19">DEC2HEX(HEX2DEC(A39)+4,8)</f>
         <v>000FE64C</v>
       </c>
-      <c r="B40" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D40" s="15" t="s">
-        <v>86</v>
+      <c r="B40" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="4" t="str">
-        <f t="shared" ref="A41" si="28">DEC2HEX(HEX2DEC(A40)+4,8)</f>
+      <c r="A41" s="9" t="str">
+        <f t="shared" ref="A41" si="20">DEC2HEX(HEX2DEC(A40)+4,8)</f>
         <v>000FE650</v>
       </c>
-      <c r="B41" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="D41" s="15"/>
+      <c r="B41" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" s="9"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="4" t="str">
-        <f t="shared" ref="A42" si="29">DEC2HEX(HEX2DEC(A41)+4,8)</f>
+      <c r="A42" s="9" t="str">
+        <f t="shared" ref="A42" si="21">DEC2HEX(HEX2DEC(A41)+4,8)</f>
         <v>000FE654</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="C42" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="15"/>
+      <c r="D42" s="9"/>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="4" t="str">
-        <f t="shared" ref="A43" si="30">DEC2HEX(HEX2DEC(A42)+4,8)</f>
+      <c r="A43" s="9" t="str">
+        <f t="shared" ref="A43" si="22">DEC2HEX(HEX2DEC(A42)+4,8)</f>
         <v>000FE658</v>
       </c>
-      <c r="B43" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="C43" s="14" t="str">
+      <c r="B43" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C43" s="8" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$54)</f>
         <v>bne 0x000FE684</v>
       </c>
-      <c r="D43" s="15"/>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" s="3" t="str">
-        <f t="shared" ref="A44" si="31">DEC2HEX(HEX2DEC(A43)+4,8)</f>
+      <c r="A44" s="6" t="str">
+        <f t="shared" ref="A44" si="23">DEC2HEX(HEX2DEC(A43)+4,8)</f>
         <v>000FE65C</v>
       </c>
-      <c r="B44" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C44" s="13" t="s">
+      <c r="B44" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D44" s="12"/>
+      <c r="D44" s="6"/>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="3" t="str">
-        <f t="shared" ref="A45" si="32">DEC2HEX(HEX2DEC(A44)+4,8)</f>
+      <c r="A45" s="6" t="str">
+        <f t="shared" ref="A45" si="24">DEC2HEX(HEX2DEC(A44)+4,8)</f>
         <v>000FE660</v>
       </c>
-      <c r="B45" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="C45" s="13" t="s">
+      <c r="B45" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C45" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="12"/>
+      <c r="D45" s="6"/>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" s="3" t="str">
-        <f t="shared" ref="A46" si="33">DEC2HEX(HEX2DEC(A45)+4,8)</f>
+      <c r="A46" s="6" t="str">
+        <f t="shared" ref="A46" si="25">DEC2HEX(HEX2DEC(A45)+4,8)</f>
         <v>000FE664</v>
       </c>
-      <c r="B46" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C46" s="13" t="s">
+      <c r="B46" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C46" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D46" s="12"/>
+      <c r="D46" s="6"/>
     </row>
     <row r="47" spans="1:4">
-      <c r="A47" s="3" t="str">
-        <f t="shared" ref="A47" si="34">DEC2HEX(HEX2DEC(A46)+4,8)</f>
+      <c r="A47" s="6" t="str">
+        <f t="shared" ref="A47" si="26">DEC2HEX(HEX2DEC(A46)+4,8)</f>
         <v>000FE668</v>
       </c>
-      <c r="B47" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C47" s="13" t="s">
+      <c r="B47" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C47" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D47" s="12"/>
+      <c r="D47" s="6"/>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" s="3" t="str">
-        <f t="shared" ref="A48" si="35">DEC2HEX(HEX2DEC(A47)+4,8)</f>
+      <c r="A48" s="6" t="str">
+        <f t="shared" ref="A48" si="27">DEC2HEX(HEX2DEC(A47)+4,8)</f>
         <v>000FE66C</v>
       </c>
-      <c r="B48" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="C48" s="13" t="s">
+      <c r="B48" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C48" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D48" s="12" t="s">
-        <v>81</v>
+      <c r="D48" s="6" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="1:4">
-      <c r="A49" s="3" t="str">
-        <f t="shared" ref="A49" si="36">DEC2HEX(HEX2DEC(A48)+4,8)</f>
+      <c r="A49" s="6" t="str">
+        <f t="shared" ref="A49" si="28">DEC2HEX(HEX2DEC(A48)+4,8)</f>
         <v>000FE670</v>
       </c>
-      <c r="B49" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C49" s="13" t="str">
+      <c r="B49" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C49" s="7" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$54)</f>
         <v>bne 0x000FE684</v>
       </c>
-      <c r="D49" s="12"/>
+      <c r="D49" s="6"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" t="str">
-        <f t="shared" ref="A50" si="37">DEC2HEX(HEX2DEC(A49)+4,8)</f>
+      <c r="A50" s="3" t="str">
+        <f t="shared" ref="A50" si="29">DEC2HEX(HEX2DEC(A49)+4,8)</f>
         <v>000FE674</v>
       </c>
-      <c r="B50" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="C50" s="8" t="str">
+      <c r="B50" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" s="2" t="str">
         <f>SUBSTITUTE(C37,"push","pop")</f>
         <v>pop {r4, r5, lr}</v>
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" t="str">
-        <f t="shared" ref="A51" si="38">DEC2HEX(HEX2DEC(A50)+4,8)</f>
+      <c r="A51" s="3" t="str">
+        <f t="shared" ref="A51" si="30">DEC2HEX(HEX2DEC(A50)+4,8)</f>
         <v>000FE678</v>
       </c>
-      <c r="B51" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="C51" s="8" t="s">
+      <c r="B51" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="3" t="str">
+        <f t="shared" ref="A52" si="31">DEC2HEX(HEX2DEC(A51)+4,8)</f>
+        <v>000FE67C</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
-      <c r="A52" t="str">
-        <f t="shared" ref="A52" si="39">DEC2HEX(HEX2DEC(A51)+4,8)</f>
-        <v>000FE67C</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="C52" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
     <row r="53" spans="1:4">
-      <c r="A53" t="str">
-        <f t="shared" ref="A53" si="40">DEC2HEX(HEX2DEC(A52)+4,8)</f>
+      <c r="A53" s="3" t="str">
+        <f t="shared" ref="A53" si="32">DEC2HEX(HEX2DEC(A52)+4,8)</f>
         <v>000FE680</v>
       </c>
-      <c r="B53" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>179</v>
+      <c r="B53" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" t="str">
-        <f t="shared" ref="A54" si="41">DEC2HEX(HEX2DEC(A53)+4,8)</f>
+      <c r="A54" s="3" t="str">
+        <f t="shared" ref="A54" si="33">DEC2HEX(HEX2DEC(A53)+4,8)</f>
         <v>000FE684</v>
       </c>
-      <c r="B54" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="C54" s="8" t="str">
+      <c r="B54" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C54" s="2" t="str">
         <f>SUBSTITUTE(C50,"lr","pc")</f>
         <v>pop {r4, r5, pc}</v>
       </c>
     </row>
     <row r="55" spans="1:4">
-      <c r="C55" s="10"/>
+      <c r="C55" s="4"/>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C56" s="10"/>
+        <v>89</v>
+      </c>
+      <c r="C56" s="4"/>
     </row>
     <row r="57" spans="1:4">
-      <c r="A57" t="str">
+      <c r="A57" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(A54)+4,8)</f>
         <v>000FE688</v>
       </c>
-      <c r="B57" s="9" t="s">
+      <c r="B57" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" t="str">
-        <f t="shared" ref="A58:A78" si="42">DEC2HEX(HEX2DEC(A57)+4,8)</f>
+      <c r="A58" s="3" t="str">
+        <f t="shared" ref="A58:A78" si="34">DEC2HEX(HEX2DEC(A57)+4,8)</f>
         <v>000FE68C</v>
       </c>
-      <c r="B58" s="9" t="s">
+      <c r="B58" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="59" spans="1:4">
-      <c r="A59" t="str">
-        <f t="shared" si="42"/>
+      <c r="A59" s="3" t="str">
+        <f t="shared" si="34"/>
         <v>000FE690</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="B59" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C59" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="60" spans="1:4">
-      <c r="A60" s="4" t="str">
-        <f t="shared" si="42"/>
+      <c r="A60" s="9" t="str">
+        <f t="shared" si="34"/>
         <v>000FE694</v>
       </c>
-      <c r="B60" s="15" t="s">
+      <c r="B60" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C60" s="14" t="s">
+      <c r="C60" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D60" s="15" t="s">
-        <v>87</v>
+      <c r="D60" s="9" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="61" spans="1:4">
-      <c r="A61" s="4" t="str">
-        <f t="shared" si="42"/>
+      <c r="A61" s="9" t="str">
+        <f t="shared" si="34"/>
         <v>000FE698</v>
       </c>
-      <c r="B61" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="C61" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="D61" s="15"/>
+      <c r="B61" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="D61" s="9"/>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="4" t="str">
-        <f t="shared" si="42"/>
+      <c r="A62" s="9" t="str">
+        <f t="shared" si="34"/>
         <v>000FE69C</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B62" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C62" s="14" t="s">
+      <c r="C62" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D62" s="15"/>
+      <c r="D62" s="9"/>
     </row>
     <row r="63" spans="1:4">
-      <c r="A63" s="4" t="str">
-        <f t="shared" si="42"/>
+      <c r="A63" s="9" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6A0</v>
       </c>
-      <c r="B63" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="C63" s="14" t="str">
+      <c r="B63" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C63" s="8" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$78)</f>
         <v>bne 0x000FE6DC</v>
       </c>
-      <c r="D63" s="15"/>
+      <c r="D63" s="9"/>
     </row>
     <row r="64" spans="1:4">
-      <c r="A64" s="3" t="str">
-        <f t="shared" si="42"/>
+      <c r="A64" s="6" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6A4</v>
       </c>
-      <c r="B64" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C64" s="13" t="s">
+      <c r="B64" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D64" s="12" t="s">
-        <v>88</v>
+      <c r="D64" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="65" spans="1:4">
-      <c r="A65" s="3" t="str">
-        <f t="shared" si="42"/>
+      <c r="A65" s="6" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6A8</v>
       </c>
-      <c r="B65" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="C65" s="13" t="s">
+      <c r="B65" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D65" s="12"/>
+      <c r="D65" s="6"/>
     </row>
     <row r="66" spans="1:4">
-      <c r="A66" s="3" t="str">
-        <f t="shared" si="42"/>
+      <c r="A66" s="6" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6AC</v>
       </c>
-      <c r="B66" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="C66" s="13" t="s">
+      <c r="B66" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C66" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D66" s="12"/>
+      <c r="D66" s="6"/>
     </row>
     <row r="67" spans="1:4">
-      <c r="A67" s="3" t="str">
-        <f t="shared" si="42"/>
+      <c r="A67" s="6" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6B0</v>
       </c>
-      <c r="B67" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="C67" s="13" t="s">
+      <c r="B67" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C67" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D67" s="12"/>
+      <c r="D67" s="6"/>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="3" t="str">
-        <f t="shared" si="42"/>
+      <c r="A68" s="6" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6B4</v>
       </c>
-      <c r="B68" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C68" s="13" t="s">
+      <c r="B68" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C68" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D68" s="12"/>
+      <c r="D68" s="6"/>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" s="3" t="str">
-        <f t="shared" si="42"/>
+      <c r="A69" s="6" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6B8</v>
       </c>
-      <c r="B69" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="C69" s="13" t="str">
+      <c r="B69" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C69" s="7" t="str">
         <f>C63</f>
         <v>bne 0x000FE6DC</v>
       </c>
-      <c r="D69" s="12"/>
+      <c r="D69" s="6"/>
     </row>
     <row r="70" spans="1:4">
-      <c r="A70" s="5" t="str">
-        <f t="shared" si="42"/>
+      <c r="A70" s="10" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6BC</v>
       </c>
-      <c r="B70" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="C70" s="17" t="s">
+      <c r="B70" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="C70" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D70" s="16" t="s">
-        <v>89</v>
+      <c r="D70" s="10" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="71" spans="1:4">
-      <c r="A71" s="5" t="str">
-        <f t="shared" si="42"/>
+      <c r="A71" s="10" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6C0</v>
       </c>
-      <c r="B71" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="C71" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="D71" s="16"/>
+      <c r="B71" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="D71" s="10"/>
     </row>
     <row r="72" spans="1:4">
-      <c r="A72" s="5" t="str">
-        <f t="shared" si="42"/>
+      <c r="A72" s="10" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6C4</v>
       </c>
-      <c r="B72" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C72" s="17" t="s">
+      <c r="B72" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C72" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D72" s="16"/>
+      <c r="D72" s="10"/>
     </row>
     <row r="73" spans="1:4">
-      <c r="A73" s="5" t="str">
-        <f t="shared" si="42"/>
+      <c r="A73" s="10" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6C8</v>
       </c>
-      <c r="B73" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="C73" s="17" t="str">
+      <c r="B73" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C73" s="11" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$78)</f>
         <v>bne 0x000FE6DC</v>
       </c>
-      <c r="D73" s="16"/>
+      <c r="D73" s="10"/>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" t="str">
-        <f t="shared" si="42"/>
+      <c r="A74" s="3" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6CC</v>
       </c>
-      <c r="B74" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="C74" s="8" t="str">
+      <c r="B74" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C74" s="2" t="str">
         <f>SUBSTITUTE(C57,"push","pop")</f>
         <v>pop {r4, r5, lr}</v>
       </c>
     </row>
     <row r="75" spans="1:4">
-      <c r="A75" t="str">
-        <f t="shared" si="42"/>
+      <c r="A75" s="3" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6D0</v>
       </c>
-      <c r="B75" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="C75" s="8" t="s">
-        <v>85</v>
+      <c r="B75" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" t="str">
-        <f t="shared" si="42"/>
+      <c r="A76" s="3" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6D4</v>
       </c>
-      <c r="B76" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="C76" s="8" t="s">
-        <v>84</v>
+      <c r="B76" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="77" spans="1:4">
-      <c r="A77" t="str">
-        <f t="shared" si="42"/>
+      <c r="A77" s="3" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6D8</v>
       </c>
-      <c r="B77" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="C77" s="8" t="s">
-        <v>179</v>
+      <c r="B77" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" t="str">
-        <f t="shared" si="42"/>
+      <c r="A78" s="3" t="str">
+        <f t="shared" si="34"/>
         <v>000FE6DC</v>
       </c>
-      <c r="B78" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="C78" s="8" t="str">
+      <c r="B78" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C78" s="2" t="str">
         <f>SUBSTITUTE(C74,"lr","pc")</f>
         <v>pop {r4, r5, pc}</v>
       </c>
     </row>
     <row r="79" spans="1:4">
-      <c r="C79" s="10"/>
+      <c r="C79" s="4"/>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="C80" s="10"/>
+        <v>181</v>
+      </c>
+      <c r="C80" s="4"/>
     </row>
     <row r="81" spans="1:6">
-      <c r="A81" t="str">
+      <c r="A81" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(A78)+4,8)</f>
         <v>000FE6E0</v>
       </c>
-      <c r="B81" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C81" s="9" t="s">
-        <v>92</v>
+      <c r="B81" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" t="str">
-        <f t="shared" ref="A82:A110" si="43">DEC2HEX(HEX2DEC(A81)+4,8)</f>
+      <c r="A82" s="3" t="str">
+        <f t="shared" ref="A82:A110" si="35">DEC2HEX(HEX2DEC(A81)+4,8)</f>
         <v>000FE6E4</v>
       </c>
-      <c r="B82" s="9" t="s">
+      <c r="B82" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C82" s="9" t="s">
+      <c r="C82" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="83" spans="1:6">
-      <c r="A83" t="str">
-        <f t="shared" si="43"/>
+      <c r="A83" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE6E8</v>
       </c>
-      <c r="B83" s="9" t="s">
+      <c r="B83" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C83" s="8" t="s">
+      <c r="C83" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="84" spans="1:6">
-      <c r="A84" s="4" t="str">
-        <f t="shared" si="43"/>
+      <c r="A84" s="9" t="str">
+        <f t="shared" si="35"/>
         <v>000FE6EC</v>
       </c>
-      <c r="B84" s="15" t="s">
+      <c r="B84" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C84" s="14" t="s">
+      <c r="C84" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D84" s="15" t="s">
-        <v>54</v>
+      <c r="D84" s="9" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="85" spans="1:6">
-      <c r="A85" s="4" t="str">
-        <f t="shared" si="43"/>
+      <c r="A85" s="9" t="str">
+        <f t="shared" si="35"/>
         <v>000FE6F0</v>
       </c>
-      <c r="B85" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="C85" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="D85" s="15"/>
+      <c r="B85" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="D85" s="9"/>
     </row>
     <row r="86" spans="1:6">
-      <c r="A86" s="4" t="str">
-        <f t="shared" si="43"/>
+      <c r="A86" s="9" t="str">
+        <f t="shared" si="35"/>
         <v>000FE6F4</v>
       </c>
-      <c r="B86" s="14" t="s">
+      <c r="B86" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C86" s="14" t="s">
+      <c r="C86" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D86" s="15"/>
+      <c r="D86" s="9"/>
     </row>
     <row r="87" spans="1:6">
-      <c r="A87" s="4" t="str">
-        <f t="shared" si="43"/>
+      <c r="A87" s="9" t="str">
+        <f t="shared" si="35"/>
         <v>000FE6F8</v>
       </c>
-      <c r="B87" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="C87" s="14" t="str">
+      <c r="B87" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C87" s="8" t="str">
         <f>_xlfn.CONCAT("beq 0x",A$92)</f>
         <v>beq 0x000FE70C</v>
       </c>
-      <c r="D87" s="15"/>
+      <c r="D87" s="9"/>
     </row>
     <row r="88" spans="1:6">
-      <c r="A88" s="3" t="str">
-        <f t="shared" ref="A88" si="44">DEC2HEX(HEX2DEC(A87)+4,8)</f>
+      <c r="A88" s="6" t="str">
+        <f t="shared" ref="A88" si="36">DEC2HEX(HEX2DEC(A87)+4,8)</f>
         <v>000FE6FC</v>
       </c>
-      <c r="B88" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C88" s="13" t="s">
+      <c r="B88" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C88" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D88" s="12" t="s">
-        <v>55</v>
+      <c r="D88" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="89" spans="1:6">
-      <c r="A89" s="3" t="str">
-        <f t="shared" ref="A89" si="45">DEC2HEX(HEX2DEC(A88)+4,8)</f>
+      <c r="A89" s="6" t="str">
+        <f t="shared" ref="A89" si="37">DEC2HEX(HEX2DEC(A88)+4,8)</f>
         <v>000FE700</v>
       </c>
-      <c r="B89" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="C89" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="D89" s="12"/>
+      <c r="B89" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D89" s="6"/>
     </row>
     <row r="90" spans="1:6">
-      <c r="A90" s="3" t="str">
-        <f t="shared" ref="A90" si="46">DEC2HEX(HEX2DEC(A89)+4,8)</f>
+      <c r="A90" s="6" t="str">
+        <f t="shared" ref="A90" si="38">DEC2HEX(HEX2DEC(A89)+4,8)</f>
         <v>000FE704</v>
       </c>
-      <c r="B90" s="13" t="s">
+      <c r="B90" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C90" s="13" t="s">
+      <c r="C90" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D90" s="12"/>
+      <c r="D90" s="6"/>
     </row>
     <row r="91" spans="1:6">
-      <c r="A91" s="3" t="str">
-        <f t="shared" ref="A91" si="47">DEC2HEX(HEX2DEC(A90)+4,8)</f>
+      <c r="A91" s="6" t="str">
+        <f t="shared" ref="A91" si="39">DEC2HEX(HEX2DEC(A90)+4,8)</f>
         <v>000FE708</v>
       </c>
-      <c r="B91" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C91" s="13" t="str">
+      <c r="B91" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="C91" s="7" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$108)</f>
         <v>bne 0x000FE74C</v>
       </c>
-      <c r="D91" s="12"/>
+      <c r="D91" s="6"/>
     </row>
     <row r="92" spans="1:6">
-      <c r="A92" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A92" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE70C</v>
       </c>
-      <c r="B92" s="16" t="s">
+      <c r="B92" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C92" s="17" t="s">
+      <c r="C92" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D92" s="16" t="s">
-        <v>58</v>
+      <c r="D92" s="10" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="93" spans="1:6">
-      <c r="A93" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A93" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE710</v>
       </c>
-      <c r="B93" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="C93" s="17" t="s">
+      <c r="B93" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C93" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="D93" s="10"/>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="10" t="str">
+        <f t="shared" si="35"/>
+        <v>000FE714</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C94" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D94" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="D93" s="16"/>
-    </row>
-    <row r="94" spans="1:6">
-      <c r="A94" s="5" t="str">
-        <f t="shared" si="43"/>
-        <v>000FE714</v>
-      </c>
-      <c r="B94" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="C94" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="D94" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="E94" t="s">
+      <c r="E94" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="95" spans="1:6">
-      <c r="A95" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A95" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE718</v>
       </c>
-      <c r="B95" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="C95" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="D95" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="E95" t="s">
+      <c r="B95" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D95" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="E95" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F95" t="s">
+      <c r="F95" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="96" spans="1:6">
-      <c r="A96" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A96" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE71C</v>
       </c>
-      <c r="B96" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="C96" s="17" t="str">
+      <c r="B96" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C96" s="11" t="str">
         <f>_xlfn.CONCAT("beq 0x",A100)</f>
         <v>beq 0x000FE72C</v>
       </c>
-      <c r="D96" s="16"/>
+      <c r="D96" s="10"/>
     </row>
     <row r="97" spans="1:7">
-      <c r="A97" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A97" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE720</v>
       </c>
-      <c r="B97" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="C97" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D97" s="16" t="s">
-        <v>189</v>
+      <c r="B97" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C97" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D97" s="10" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="98" spans="1:7">
-      <c r="A98" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A98" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE724</v>
       </c>
-      <c r="B98" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="C98" s="17" t="str">
+      <c r="B98" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C98" s="11" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$108)</f>
         <v>bne 0x000FE74C</v>
       </c>
-      <c r="D98" s="16"/>
+      <c r="D98" s="10"/>
     </row>
     <row r="99" spans="1:7">
-      <c r="A99" s="5" t="str">
-        <f t="shared" si="43"/>
+      <c r="A99" s="10" t="str">
+        <f t="shared" si="35"/>
         <v>000FE728</v>
       </c>
-      <c r="B99" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="C99" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D99" s="16" t="s">
-        <v>191</v>
+      <c r="B99" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="C99" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D99" s="10" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="100" spans="1:7">
-      <c r="A100" t="str">
-        <f t="shared" si="43"/>
+      <c r="A100" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE72C</v>
       </c>
-      <c r="B100" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="C100" s="8" t="str">
+      <c r="B100" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C100" s="2" t="str">
         <f>_xlfn.CONCAT("ldr r7, [pc, 0x",DEC2HEX(HEX2DEC(A110)-HEX2DEC(A100)-8,3),"]")</f>
         <v>ldr r7, [pc, 0x020]</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="D100" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7">
+      <c r="A101" s="3" t="str">
+        <f t="shared" si="35"/>
+        <v>000FE730</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7">
+      <c r="A102" s="3" t="str">
+        <f t="shared" si="35"/>
+        <v>000FE734</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C102" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="101" spans="1:7">
-      <c r="A101" t="str">
-        <f t="shared" si="43"/>
-        <v>000FE730</v>
-      </c>
-      <c r="B101" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="C101" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="D101" s="9" t="s">
+      <c r="D102" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
-      <c r="A102" t="str">
-        <f t="shared" si="43"/>
-        <v>000FE734</v>
-      </c>
-      <c r="B102" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C102" s="8" t="s">
+    <row r="103" spans="1:7">
+      <c r="A103" s="3" t="str">
+        <f t="shared" si="35"/>
+        <v>000FE738</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C103" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D102" s="9" t="s">
+      <c r="D103" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
-      <c r="A103" t="str">
-        <f t="shared" si="43"/>
-        <v>000FE738</v>
-      </c>
-      <c r="B103" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C103" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D103" s="9" t="s">
-        <v>63</v>
-      </c>
-    </row>
     <row r="104" spans="1:7">
-      <c r="A104" t="str">
-        <f t="shared" si="43"/>
+      <c r="A104" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE73C</v>
       </c>
-      <c r="B104" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="C104" s="8" t="s">
-        <v>171</v>
+      <c r="B104" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="105" spans="1:7">
-      <c r="A105" t="str">
-        <f t="shared" si="43"/>
+      <c r="A105" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE740</v>
       </c>
-      <c r="B105" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="C105" s="8" t="str">
+      <c r="B105" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C105" s="2" t="str">
         <f>_xlfn.CONCAT("bhs 0x",A$108)</f>
         <v>bhs 0x000FE74C</v>
       </c>
-      <c r="D105" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="F105" t="s">
-        <v>65</v>
+      <c r="D105" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="106" spans="1:7">
-      <c r="A106" t="str">
-        <f t="shared" si="43"/>
+      <c r="A106" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE744</v>
       </c>
-      <c r="B106" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="C106" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F106" t="s">
+      <c r="B106" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7">
+      <c r="A107" s="3" t="str">
+        <f t="shared" si="35"/>
+        <v>000FE748</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F107" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="107" spans="1:7">
-      <c r="A107" t="str">
-        <f t="shared" si="43"/>
-        <v>000FE748</v>
-      </c>
-      <c r="B107" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C107" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F107" t="s">
-        <v>68</v>
-      </c>
-    </row>
     <row r="108" spans="1:7">
-      <c r="A108" t="str">
-        <f t="shared" si="43"/>
+      <c r="A108" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE74C</v>
       </c>
-      <c r="B108" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="C108" s="8" t="str">
+      <c r="B108" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C108" s="2" t="str">
         <f>SUBSTITUTE(C81,"push","pop")</f>
         <v>pop {r4, r5, r6, r7, lr}</v>
       </c>
-      <c r="F108" t="s">
-        <v>66</v>
+      <c r="F108" s="3" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="109" spans="1:7">
-      <c r="A109" t="str">
-        <f t="shared" si="43"/>
+      <c r="A109" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE750</v>
       </c>
-      <c r="B109" s="9" t="s">
+      <c r="B109" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C109" s="8" t="s">
+      <c r="C109" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F109" t="s">
-        <v>69</v>
+      <c r="F109" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="110" spans="1:7">
-      <c r="A110" t="str">
-        <f t="shared" si="43"/>
+      <c r="A110" s="3" t="str">
+        <f t="shared" si="35"/>
         <v>000FE754</v>
       </c>
-      <c r="B110" s="8" t="s">
+      <c r="B110" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C110" s="9" t="s">
+      <c r="C110" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F110" t="s">
-        <v>64</v>
-      </c>
-      <c r="G110" t="str">
+      <c r="F110" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G110" s="3" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,F105:F110)</f>
         <v>Apex Bulbasaur, Electivire, Magmortar, Heatran, Rotom-H, Mega Togedemaru</v>
       </c>
     </row>
     <row r="112" spans="1:7">
-      <c r="C112" s="10"/>
+      <c r="C112" s="4"/>
     </row>
     <row r="113" spans="1:5">
       <c r="A113" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C113" s="10"/>
+        <v>70</v>
+      </c>
+      <c r="C113" s="4"/>
     </row>
     <row r="114" spans="1:5">
-      <c r="A114" t="str">
+      <c r="A114" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(A110)+4,8)</f>
         <v>000FE758</v>
       </c>
-      <c r="B114" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C114" s="9" t="s">
-        <v>92</v>
+      <c r="B114" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="115" spans="1:5">
-      <c r="A115" t="str">
-        <f t="shared" ref="A115:A148" si="48">DEC2HEX(HEX2DEC(A114)+4,8)</f>
+      <c r="A115" s="3" t="str">
+        <f t="shared" ref="A115:A148" si="40">DEC2HEX(HEX2DEC(A114)+4,8)</f>
         <v>000FE75C</v>
       </c>
-      <c r="B115" s="9" t="s">
+      <c r="B115" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C115" s="9" t="s">
+      <c r="C115" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="116" spans="1:5">
-      <c r="A116" t="str">
-        <f t="shared" si="48"/>
+      <c r="A116" s="3" t="str">
+        <f t="shared" si="40"/>
         <v>000FE760</v>
       </c>
-      <c r="B116" s="9" t="s">
+      <c r="B116" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C116" s="8" t="s">
+      <c r="C116" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="117" spans="1:5">
-      <c r="A117" s="4" t="str">
-        <f t="shared" si="48"/>
+      <c r="A117" s="9" t="str">
+        <f t="shared" si="40"/>
         <v>000FE764</v>
       </c>
-      <c r="B117" s="15" t="s">
+      <c r="B117" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C117" s="14" t="s">
+      <c r="C117" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D117" s="15" t="s">
-        <v>54</v>
+      <c r="D117" s="9" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="118" spans="1:5">
-      <c r="A118" s="4" t="str">
-        <f t="shared" si="48"/>
+      <c r="A118" s="9" t="str">
+        <f t="shared" si="40"/>
         <v>000FE768</v>
       </c>
-      <c r="B118" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="C118" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="D118" s="15"/>
+      <c r="B118" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C118" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="D118" s="9"/>
     </row>
     <row r="119" spans="1:5">
-      <c r="A119" s="4" t="str">
-        <f t="shared" si="48"/>
+      <c r="A119" s="9" t="str">
+        <f t="shared" si="40"/>
         <v>000FE76C</v>
       </c>
-      <c r="B119" s="14" t="s">
+      <c r="B119" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C119" s="14" t="s">
+      <c r="C119" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D119" s="15"/>
+      <c r="D119" s="9"/>
     </row>
     <row r="120" spans="1:5">
-      <c r="A120" s="4" t="str">
-        <f t="shared" si="48"/>
+      <c r="A120" s="9" t="str">
+        <f t="shared" si="40"/>
         <v>000FE770</v>
       </c>
-      <c r="B120" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="C120" s="14" t="str">
+      <c r="B120" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C120" s="8" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$147)</f>
         <v>bne 0x000FE7DC</v>
       </c>
-      <c r="D120" s="15"/>
+      <c r="D120" s="9"/>
     </row>
     <row r="121" spans="1:5">
-      <c r="A121" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A121" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE774</v>
       </c>
-      <c r="B121" s="12" t="s">
+      <c r="B121" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C121" s="13" t="s">
+      <c r="C121" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D121" s="12" t="s">
-        <v>58</v>
+      <c r="D121" s="6" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="122" spans="1:5">
-      <c r="A122" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A122" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE778</v>
       </c>
-      <c r="B122" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="C122" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="D122" s="12"/>
+      <c r="B122" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D122" s="6"/>
     </row>
     <row r="123" spans="1:5">
-      <c r="A123" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A123" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE77C</v>
       </c>
-      <c r="B123" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="C123" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="D123" s="12" t="s">
-        <v>192</v>
-      </c>
-      <c r="E123" t="s">
-        <v>181</v>
+      <c r="B123" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D123" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="124" spans="1:5">
-      <c r="A124" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A124" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE780</v>
       </c>
-      <c r="B124" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="C124" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="D124" s="12" t="s">
-        <v>191</v>
+      <c r="B124" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D124" s="6" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="125" spans="1:5">
-      <c r="A125" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A125" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE784</v>
       </c>
-      <c r="B125" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C125" s="13" t="str">
+      <c r="B125" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C125" s="7" t="str">
         <f>_xlfn.CONCAT("beq 0x",A129)</f>
         <v>beq 0x000FE794</v>
       </c>
-      <c r="D125" s="12"/>
+      <c r="D125" s="6"/>
     </row>
     <row r="126" spans="1:5">
-      <c r="A126" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A126" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE788</v>
       </c>
-      <c r="B126" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="C126" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D126" s="12" t="s">
-        <v>195</v>
+      <c r="B126" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D126" s="6" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="127" spans="1:5">
-      <c r="A127" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A127" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE78C</v>
       </c>
-      <c r="B127" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="C127" s="13" t="str">
+      <c r="B127" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C127" s="7" t="str">
         <f>_xlfn.CONCAT("bne 0x",A$147)</f>
         <v>bne 0x000FE7DC</v>
       </c>
-      <c r="D127" s="12"/>
+      <c r="D127" s="6"/>
     </row>
     <row r="128" spans="1:5">
-      <c r="A128" s="3" t="str">
-        <f t="shared" si="48"/>
+      <c r="A128" s="6" t="str">
+        <f t="shared" si="40"/>
         <v>000FE790</v>
       </c>
-      <c r="B128" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="C128" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="D128" s="12" t="s">
-        <v>190</v>
+      <c r="B128" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C128" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D128" s="6" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="129" spans="1:4">
-      <c r="A129" s="5" t="str">
-        <f t="shared" si="48"/>
+      <c r="A129" s="10" t="str">
+        <f t="shared" si="40"/>
         <v>000FE794</v>
       </c>
-      <c r="B129" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="C129" s="17" t="str">
+      <c r="B129" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C129" s="11" t="str">
         <f>_xlfn.CONCAT("ldr r7, [pc, 0x",DEC2HEX(HEX2DEC(A148)-HEX2DEC(A129)-8,3),"]")</f>
         <v>ldr r7, [pc, 0x044]</v>
       </c>
-      <c r="D129" s="16" t="s">
-        <v>93</v>
+      <c r="D129" s="10" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="130" spans="1:4">
-      <c r="A130" s="5" t="str">
-        <f t="shared" si="48"/>
+      <c r="A130" s="10" t="str">
+        <f t="shared" si="40"/>
         <v>000FE798</v>
       </c>
-      <c r="B130" s="17" t="s">
+      <c r="B130" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C130" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D130" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" s="10" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE79C</v>
+      </c>
+      <c r="B131" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C131" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D131" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" s="10" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7A0</v>
+      </c>
+      <c r="B132" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="C132" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D132" s="10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7A4</v>
+      </c>
+      <c r="B133" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C133" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D133" s="13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7A8</v>
+      </c>
+      <c r="B134" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C134" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D134" s="13"/>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7AC</v>
+      </c>
+      <c r="B135" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C135" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D135" s="13"/>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7B0</v>
+      </c>
+      <c r="B136" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C136" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D136" s="13"/>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7B4</v>
+      </c>
+      <c r="B137" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C137" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D137" s="13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7B8</v>
+      </c>
+      <c r="B138" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C138" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D138" s="13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="13" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7BC</v>
+      </c>
+      <c r="B139" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="C139" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="D139" s="13"/>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="3" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7C0</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="3" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7C4</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="3" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7C8</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="3" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7CC</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
+      <c r="A144" s="3" t="str">
+        <f t="shared" si="40"/>
+        <v>000FE7D0</v>
+      </c>
+      <c r="B144" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C130" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D130" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4">
-      <c r="A131" s="5" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE79C</v>
-      </c>
-      <c r="B131" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="C131" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="D131" s="16" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4">
-      <c r="A132" s="5" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7A0</v>
-      </c>
-      <c r="B132" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="C132" s="17" t="s">
-        <v>174</v>
-      </c>
-      <c r="D132" s="16" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4">
-      <c r="A133" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7A4</v>
-      </c>
-      <c r="B133" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="C133" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="D133" s="19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4">
-      <c r="A134" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7A8</v>
-      </c>
-      <c r="B134" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="C134" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="D134" s="19"/>
-    </row>
-    <row r="135" spans="1:4">
-      <c r="A135" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7AC</v>
-      </c>
-      <c r="B135" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="C135" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D135" s="19"/>
-    </row>
-    <row r="136" spans="1:4">
-      <c r="A136" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7B0</v>
-      </c>
-      <c r="B136" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="C136" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="D136" s="19"/>
-    </row>
-    <row r="137" spans="1:4">
-      <c r="A137" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7B4</v>
-      </c>
-      <c r="B137" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="C137" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="D137" s="19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4">
-      <c r="A138" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7B8</v>
-      </c>
-      <c r="B138" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="C138" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="D138" s="19" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4">
-      <c r="A139" s="6" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7BC</v>
-      </c>
-      <c r="B139" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="C139" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="D139" s="19"/>
-    </row>
-    <row r="140" spans="1:4">
-      <c r="A140" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7C0</v>
-      </c>
-      <c r="B140" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="C140" s="8" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4">
-      <c r="A141" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7C4</v>
-      </c>
-      <c r="B141" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="C141" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="D141" s="9" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4">
-      <c r="A142" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7C8</v>
-      </c>
-      <c r="B142" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C142" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4">
-      <c r="A143" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7CC</v>
-      </c>
-      <c r="B143" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="C143" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D143" s="9" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4">
-      <c r="A144" t="str">
-        <f t="shared" si="48"/>
-        <v>000FE7D0</v>
-      </c>
-      <c r="B144" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="C144" s="8" t="str">
+      <c r="C144" s="2" t="str">
         <f>SUBSTITUTE(C114,"push","pop")</f>
         <v>pop {r4, r5, r6, r7, lr}</v>
       </c>
     </row>
     <row r="145" spans="1:9">
-      <c r="A145" t="str">
-        <f t="shared" si="48"/>
+      <c r="A145" s="3" t="str">
+        <f t="shared" si="40"/>
         <v>000FE7D4</v>
       </c>
-      <c r="B145" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="C145" s="9" t="s">
+      <c r="B145" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C145" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="146" spans="1:9">
-      <c r="A146" t="str">
-        <f t="shared" si="48"/>
+      <c r="A146" s="3" t="str">
+        <f t="shared" si="40"/>
         <v>000FE7D8</v>
       </c>
-      <c r="B146" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="C146" s="8" t="s">
-        <v>180</v>
+      <c r="B146" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="147" spans="1:9">
-      <c r="A147" t="str">
-        <f t="shared" si="48"/>
+      <c r="A147" s="3" t="str">
+        <f t="shared" si="40"/>
         <v>000FE7DC</v>
       </c>
-      <c r="B147" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="C147" s="9" t="str">
+      <c r="B147" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C147" s="3" t="str">
         <f>SUBSTITUTE(C144,"lr","pc")</f>
         <v>pop {r4, r5, r6, r7, pc}</v>
       </c>
     </row>
     <row r="148" spans="1:9">
-      <c r="A148" t="str">
-        <f t="shared" si="48"/>
+      <c r="A148" s="3" t="str">
+        <f t="shared" si="40"/>
         <v>000FE7E0</v>
       </c>
-      <c r="B148" s="8" t="s">
+      <c r="B148" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C148" s="9" t="s">
+      <c r="C148" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="149" spans="1:9">
-      <c r="F149">
+      <c r="F149" s="3">
         <v>0</v>
       </c>
-      <c r="G149">
+      <c r="G149" s="3">
         <v>0</v>
       </c>
-      <c r="H149">
+      <c r="H149" s="3">
         <v>0</v>
       </c>
-      <c r="I149">
+      <c r="I149" s="3">
         <f>1+G149/4096</f>
         <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:9">
-      <c r="F150">
+      <c r="F150" s="3">
         <v>1</v>
       </c>
-      <c r="G150">
+      <c r="G150" s="3">
         <f>F150*128</f>
         <v>128</v>
       </c>
-      <c r="H150" t="str">
+      <c r="H150" s="3" t="str">
         <f>DEC2HEX(G150)</f>
         <v>80</v>
       </c>
-      <c r="I150">
-        <f t="shared" ref="I150:I173" si="49">1+G150/4096</f>
+      <c r="I150" s="3">
+        <f t="shared" ref="I150:I173" si="41">1+G150/4096</f>
         <v>1.03125</v>
       </c>
     </row>
     <row r="151" spans="1:9">
-      <c r="F151">
+      <c r="F151" s="3">
         <f>F150+1</f>
         <v>2</v>
       </c>
-      <c r="G151">
+      <c r="G151" s="3">
         <f>F151*128</f>
         <v>256</v>
       </c>
-      <c r="H151" t="str">
-        <f t="shared" ref="H151:H173" si="50">DEC2HEX(G151)</f>
+      <c r="H151" s="3" t="str">
+        <f t="shared" ref="H151:H173" si="42">DEC2HEX(G151)</f>
         <v>100</v>
       </c>
-      <c r="I151">
-        <f t="shared" si="49"/>
+      <c r="I151" s="3">
+        <f t="shared" si="41"/>
         <v>1.0625</v>
       </c>
     </row>
     <row r="152" spans="1:9">
-      <c r="F152">
-        <f t="shared" ref="F152:F164" si="51">F151+1</f>
+      <c r="F152" s="3">
+        <f t="shared" ref="F152:F164" si="43">F151+1</f>
         <v>3</v>
       </c>
-      <c r="G152">
-        <f t="shared" ref="G152:G172" si="52">F152*128</f>
+      <c r="G152" s="3">
+        <f t="shared" ref="G152:G172" si="44">F152*128</f>
         <v>384</v>
       </c>
-      <c r="H152" t="str">
-        <f t="shared" si="50"/>
+      <c r="H152" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>180</v>
       </c>
-      <c r="I152">
-        <f t="shared" si="49"/>
+      <c r="I152" s="3">
+        <f t="shared" si="41"/>
         <v>1.09375</v>
       </c>
     </row>
     <row r="153" spans="1:9">
-      <c r="F153">
-        <f t="shared" si="51"/>
+      <c r="F153" s="3">
+        <f t="shared" si="43"/>
         <v>4</v>
       </c>
-      <c r="G153">
-        <f t="shared" si="52"/>
+      <c r="G153" s="3">
+        <f t="shared" si="44"/>
         <v>512</v>
       </c>
-      <c r="H153" t="str">
-        <f t="shared" si="50"/>
+      <c r="H153" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>200</v>
       </c>
-      <c r="I153">
-        <f t="shared" si="49"/>
+      <c r="I153" s="3">
+        <f t="shared" si="41"/>
         <v>1.125</v>
       </c>
     </row>
     <row r="154" spans="1:9">
-      <c r="F154">
-        <f t="shared" si="51"/>
+      <c r="F154" s="3">
+        <f t="shared" si="43"/>
         <v>5</v>
       </c>
-      <c r="G154">
-        <f t="shared" si="52"/>
+      <c r="G154" s="3">
+        <f t="shared" si="44"/>
         <v>640</v>
       </c>
-      <c r="H154" t="str">
-        <f t="shared" si="50"/>
+      <c r="H154" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>280</v>
       </c>
-      <c r="I154">
-        <f t="shared" si="49"/>
+      <c r="I154" s="3">
+        <f t="shared" si="41"/>
         <v>1.15625</v>
       </c>
     </row>
     <row r="155" spans="1:9">
-      <c r="F155">
-        <f t="shared" si="51"/>
+      <c r="F155" s="3">
+        <f t="shared" si="43"/>
         <v>6</v>
       </c>
-      <c r="G155">
-        <f t="shared" si="52"/>
+      <c r="G155" s="3">
+        <f t="shared" si="44"/>
         <v>768</v>
       </c>
-      <c r="H155" t="str">
-        <f t="shared" si="50"/>
+      <c r="H155" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>300</v>
       </c>
-      <c r="I155">
-        <f t="shared" si="49"/>
+      <c r="I155" s="3">
+        <f t="shared" si="41"/>
         <v>1.1875</v>
       </c>
     </row>
     <row r="156" spans="1:9">
-      <c r="F156">
-        <f t="shared" si="51"/>
+      <c r="F156" s="3">
+        <f t="shared" si="43"/>
         <v>7</v>
       </c>
-      <c r="G156">
-        <f t="shared" si="52"/>
+      <c r="G156" s="3">
+        <f t="shared" si="44"/>
         <v>896</v>
       </c>
-      <c r="H156" t="str">
-        <f t="shared" si="50"/>
+      <c r="H156" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>380</v>
       </c>
-      <c r="I156">
-        <f t="shared" si="49"/>
+      <c r="I156" s="3">
+        <f t="shared" si="41"/>
         <v>1.21875</v>
       </c>
     </row>
     <row r="157" spans="1:9">
-      <c r="F157">
-        <f t="shared" si="51"/>
+      <c r="F157" s="3">
+        <f t="shared" si="43"/>
         <v>8</v>
       </c>
-      <c r="G157">
-        <f t="shared" si="52"/>
+      <c r="G157" s="3">
+        <f t="shared" si="44"/>
         <v>1024</v>
       </c>
-      <c r="H157" t="str">
-        <f t="shared" si="50"/>
+      <c r="H157" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>400</v>
       </c>
-      <c r="I157">
-        <f t="shared" si="49"/>
+      <c r="I157" s="3">
+        <f t="shared" si="41"/>
         <v>1.25</v>
       </c>
     </row>
     <row r="158" spans="1:9">
-      <c r="F158">
-        <f t="shared" si="51"/>
+      <c r="F158" s="3">
+        <f t="shared" si="43"/>
         <v>9</v>
       </c>
-      <c r="G158">
-        <f t="shared" si="52"/>
+      <c r="G158" s="3">
+        <f t="shared" si="44"/>
         <v>1152</v>
       </c>
-      <c r="H158" t="str">
-        <f t="shared" si="50"/>
+      <c r="H158" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>480</v>
       </c>
-      <c r="I158">
-        <f t="shared" si="49"/>
+      <c r="I158" s="3">
+        <f t="shared" si="41"/>
         <v>1.28125</v>
       </c>
     </row>
     <row r="159" spans="1:9">
-      <c r="F159">
-        <f t="shared" si="51"/>
+      <c r="F159" s="3">
+        <f t="shared" si="43"/>
         <v>10</v>
       </c>
-      <c r="G159">
-        <f t="shared" si="52"/>
+      <c r="G159" s="3">
+        <f t="shared" si="44"/>
         <v>1280</v>
       </c>
-      <c r="H159" t="str">
-        <f t="shared" si="50"/>
+      <c r="H159" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>500</v>
       </c>
-      <c r="I159">
-        <f t="shared" si="49"/>
+      <c r="I159" s="3">
+        <f t="shared" si="41"/>
         <v>1.3125</v>
       </c>
     </row>
     <row r="160" spans="1:9">
-      <c r="F160">
-        <f t="shared" si="51"/>
+      <c r="F160" s="3">
+        <f t="shared" si="43"/>
         <v>11</v>
       </c>
-      <c r="G160">
-        <f t="shared" si="52"/>
+      <c r="G160" s="3">
+        <f t="shared" si="44"/>
         <v>1408</v>
       </c>
-      <c r="H160" t="str">
-        <f t="shared" si="50"/>
+      <c r="H160" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>580</v>
       </c>
-      <c r="I160">
-        <f t="shared" si="49"/>
+      <c r="I160" s="3">
+        <f t="shared" si="41"/>
         <v>1.34375</v>
       </c>
     </row>
     <row r="161" spans="6:9">
-      <c r="F161">
-        <f t="shared" si="51"/>
+      <c r="F161" s="3">
+        <f t="shared" si="43"/>
         <v>12</v>
       </c>
-      <c r="G161">
-        <f t="shared" si="52"/>
+      <c r="G161" s="3">
+        <f t="shared" si="44"/>
         <v>1536</v>
       </c>
-      <c r="H161" t="str">
-        <f t="shared" si="50"/>
+      <c r="H161" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>600</v>
       </c>
-      <c r="I161">
-        <f t="shared" si="49"/>
+      <c r="I161" s="3">
+        <f t="shared" si="41"/>
         <v>1.375</v>
       </c>
     </row>
     <row r="162" spans="6:9">
-      <c r="F162">
-        <f t="shared" si="51"/>
+      <c r="F162" s="3">
+        <f t="shared" si="43"/>
         <v>13</v>
       </c>
-      <c r="G162">
-        <f t="shared" si="52"/>
+      <c r="G162" s="3">
+        <f t="shared" si="44"/>
         <v>1664</v>
       </c>
-      <c r="H162" t="str">
-        <f t="shared" si="50"/>
+      <c r="H162" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>680</v>
       </c>
-      <c r="I162">
-        <f t="shared" si="49"/>
+      <c r="I162" s="3">
+        <f t="shared" si="41"/>
         <v>1.40625</v>
       </c>
     </row>
     <row r="163" spans="6:9">
-      <c r="F163">
-        <f t="shared" si="51"/>
+      <c r="F163" s="3">
+        <f t="shared" si="43"/>
         <v>14</v>
       </c>
-      <c r="G163">
-        <f t="shared" si="52"/>
+      <c r="G163" s="3">
+        <f t="shared" si="44"/>
         <v>1792</v>
       </c>
-      <c r="H163" t="str">
-        <f t="shared" si="50"/>
+      <c r="H163" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>700</v>
       </c>
-      <c r="I163">
-        <f t="shared" si="49"/>
+      <c r="I163" s="3">
+        <f t="shared" si="41"/>
         <v>1.4375</v>
       </c>
     </row>
     <row r="164" spans="6:9">
-      <c r="F164">
-        <f t="shared" si="51"/>
+      <c r="F164" s="3">
+        <f t="shared" si="43"/>
         <v>15</v>
       </c>
-      <c r="G164">
-        <f t="shared" si="52"/>
+      <c r="G164" s="3">
+        <f t="shared" si="44"/>
         <v>1920</v>
       </c>
-      <c r="H164" t="str">
-        <f t="shared" si="50"/>
+      <c r="H164" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>780</v>
       </c>
-      <c r="I164">
-        <f t="shared" si="49"/>
+      <c r="I164" s="3">
+        <f t="shared" si="41"/>
         <v>1.46875</v>
       </c>
     </row>
     <row r="165" spans="6:9">
-      <c r="F165">
+      <c r="F165" s="3">
         <f>F164+1</f>
         <v>16</v>
       </c>
-      <c r="G165">
+      <c r="G165" s="3">
         <f>F165*128</f>
         <v>2048</v>
       </c>
-      <c r="H165" t="str">
-        <f t="shared" si="50"/>
+      <c r="H165" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>800</v>
       </c>
-      <c r="I165">
-        <f t="shared" si="49"/>
+      <c r="I165" s="3">
+        <f t="shared" si="41"/>
         <v>1.5</v>
       </c>
     </row>
     <row r="166" spans="6:9">
-      <c r="F166">
-        <f t="shared" ref="F166:F172" si="53">F165+1</f>
+      <c r="F166" s="3">
+        <f t="shared" ref="F166:F172" si="45">F165+1</f>
         <v>17</v>
       </c>
-      <c r="G166">
-        <f t="shared" si="52"/>
+      <c r="G166" s="3">
+        <f t="shared" si="44"/>
         <v>2176</v>
       </c>
-      <c r="H166" t="str">
-        <f t="shared" si="50"/>
+      <c r="H166" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>880</v>
       </c>
-      <c r="I166">
-        <f t="shared" si="49"/>
+      <c r="I166" s="3">
+        <f t="shared" si="41"/>
         <v>1.53125</v>
       </c>
     </row>
     <row r="167" spans="6:9">
-      <c r="F167">
-        <f t="shared" si="53"/>
+      <c r="F167" s="3">
+        <f t="shared" si="45"/>
         <v>18</v>
       </c>
-      <c r="G167">
-        <f t="shared" si="52"/>
+      <c r="G167" s="3">
+        <f t="shared" si="44"/>
         <v>2304</v>
       </c>
-      <c r="H167" t="str">
-        <f t="shared" si="50"/>
+      <c r="H167" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>900</v>
       </c>
-      <c r="I167">
-        <f t="shared" si="49"/>
+      <c r="I167" s="3">
+        <f t="shared" si="41"/>
         <v>1.5625</v>
       </c>
     </row>
     <row r="168" spans="6:9">
-      <c r="F168">
-        <f t="shared" si="53"/>
+      <c r="F168" s="3">
+        <f t="shared" si="45"/>
         <v>19</v>
       </c>
-      <c r="G168">
-        <f t="shared" si="52"/>
+      <c r="G168" s="3">
+        <f t="shared" si="44"/>
         <v>2432</v>
       </c>
-      <c r="H168" t="str">
-        <f t="shared" si="50"/>
+      <c r="H168" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>980</v>
       </c>
-      <c r="I168">
-        <f t="shared" si="49"/>
+      <c r="I168" s="3">
+        <f t="shared" si="41"/>
         <v>1.59375</v>
       </c>
     </row>
     <row r="169" spans="6:9">
-      <c r="F169">
-        <f t="shared" si="53"/>
+      <c r="F169" s="3">
+        <f t="shared" si="45"/>
         <v>20</v>
       </c>
-      <c r="G169">
-        <f t="shared" si="52"/>
+      <c r="G169" s="3">
+        <f t="shared" si="44"/>
         <v>2560</v>
       </c>
-      <c r="H169" t="str">
-        <f t="shared" si="50"/>
+      <c r="H169" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>A00</v>
       </c>
-      <c r="I169">
-        <f t="shared" si="49"/>
+      <c r="I169" s="3">
+        <f t="shared" si="41"/>
         <v>1.625</v>
       </c>
     </row>
     <row r="170" spans="6:9">
-      <c r="F170">
-        <f t="shared" si="53"/>
+      <c r="F170" s="3">
+        <f t="shared" si="45"/>
         <v>21</v>
       </c>
-      <c r="G170">
-        <f t="shared" si="52"/>
+      <c r="G170" s="3">
+        <f t="shared" si="44"/>
         <v>2688</v>
       </c>
-      <c r="H170" t="str">
-        <f t="shared" si="50"/>
+      <c r="H170" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>A80</v>
       </c>
-      <c r="I170">
-        <f t="shared" si="49"/>
+      <c r="I170" s="3">
+        <f t="shared" si="41"/>
         <v>1.65625</v>
       </c>
     </row>
     <row r="171" spans="6:9">
-      <c r="F171">
-        <f t="shared" si="53"/>
+      <c r="F171" s="3">
+        <f t="shared" si="45"/>
         <v>22</v>
       </c>
-      <c r="G171">
-        <f t="shared" si="52"/>
+      <c r="G171" s="3">
+        <f t="shared" si="44"/>
         <v>2816</v>
       </c>
-      <c r="H171" t="str">
-        <f t="shared" si="50"/>
+      <c r="H171" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>B00</v>
       </c>
-      <c r="I171">
-        <f t="shared" si="49"/>
+      <c r="I171" s="3">
+        <f t="shared" si="41"/>
         <v>1.6875</v>
       </c>
     </row>
     <row r="172" spans="6:9">
-      <c r="F172">
-        <f t="shared" si="53"/>
+      <c r="F172" s="3">
+        <f t="shared" si="45"/>
         <v>23</v>
       </c>
-      <c r="G172">
-        <f t="shared" si="52"/>
+      <c r="G172" s="3">
+        <f t="shared" si="44"/>
         <v>2944</v>
       </c>
-      <c r="H172" t="str">
-        <f t="shared" si="50"/>
+      <c r="H172" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>B80</v>
       </c>
-      <c r="I172">
-        <f t="shared" si="49"/>
+      <c r="I172" s="3">
+        <f t="shared" si="41"/>
         <v>1.71875</v>
       </c>
     </row>
     <row r="173" spans="6:9">
-      <c r="F173">
+      <c r="F173" s="3">
         <f>F172+1</f>
         <v>24</v>
       </c>
-      <c r="G173">
+      <c r="G173" s="3">
         <f>F173*128</f>
         <v>3072</v>
       </c>
-      <c r="H173" t="str">
-        <f t="shared" si="50"/>
+      <c r="H173" s="3" t="str">
+        <f t="shared" si="42"/>
         <v>C00</v>
       </c>
-      <c r="I173">
-        <f t="shared" si="49"/>
+      <c r="I173" s="3">
+        <f t="shared" si="41"/>
         <v>1.75</v>
       </c>
     </row>
@@ -3537,7 +3533,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1">
         <f>LEN(A1)</f>
@@ -3546,7 +3542,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2">
         <f>LEN(A2)</f>

</xml_diff>